<commit_message>
data: hourly update 2026-07-16 15:09Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-16.xlsx
+++ b/data/output/workbook/2026-07-16.xlsx
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 01:50</t>
+          <t>2026-07-16 11:08</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5017,12 +5017,12 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -5032,17 +5032,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox +1.5</t>
+          <t>Pittsburgh Pirates +1.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.632</v>
+        <v>0.6574</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-172</v>
+        <v>-192</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 63.2% (fair -172). Your call.</t>
+          <t>Model 65.7% (fair -192). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5078,17 +5078,17 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -5098,17 +5098,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>New York Mets +1.5</t>
+          <t>Chicago White Sox +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6368</v>
+        <v>0.6302</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-175</v>
+        <v>-170</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 63.7% (fair -175). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5168,10 +5168,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6535</v>
+        <v>0.6559</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-189</v>
+        <v>-191</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 65.3% (fair -189). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5234,10 +5234,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.649</v>
+        <v>0.6299</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-185</v>
+        <v>-170</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>100</v>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 64.9% (fair -185). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5276,17 +5276,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -5296,17 +5296,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.6058</v>
+        <v>0.6077</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-154</v>
+        <v>-155</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 60.6% (fair -154). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -5342,17 +5342,17 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -5362,17 +5362,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6086</v>
+        <v>0.6064000000000001</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-155</v>
+        <v>-154</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -155). Your call.</t>
+          <t>Model 60.6% (fair -154). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -5413,12 +5413,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -5428,17 +5428,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5702</v>
+        <v>0.598</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-133</v>
+        <v>-149</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -133). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -5498,13 +5498,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5842000000000001</v>
+        <v>0.5848</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>-141</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 58.4% (fair -141). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -5560,17 +5560,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +7.5</t>
+          <t>Toronto Tempo +6.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5643</v>
+        <v>0.542</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-130</v>
+        <v>-118</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -130). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -5611,32 +5611,32 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Dallas Wings</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5653</v>
+        <v>0.4813</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-130</v>
+        <v>108</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-113</v>
+        <v>126</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -5677,32 +5677,32 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5399</v>
+        <v>0.3905</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-117</v>
+        <v>156</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-105</v>
+        <v>178</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 39.1% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -5743,32 +5743,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4001</v>
+        <v>0.3888</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 40.0% (fair +150). Your call.</t>
+          <t>Model 38.9% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -5809,32 +5809,32 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Over 183.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4936</v>
+        <v>0.5482</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>103</v>
+        <v>-121</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>113</v>
+        <v>-105</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +103). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -5870,17 +5870,17 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>New York Liberty @ Dallas Wings</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -5890,17 +5890,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Dallas Wings</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5611</v>
+        <v>0.5714</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-128</v>
+        <v>-133</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-117</v>
+        <v>-115</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -5941,32 +5941,32 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 181.5</t>
+          <t>Connecticut Sun +5.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.53</v>
+        <v>0.5134000000000001</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-113</v>
+        <v>-106</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-105</v>
+        <v>108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 51.3% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -6007,32 +6007,32 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5064</v>
+        <v>0.5503</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-103</v>
+        <v>-122</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>104</v>
+        <v>-108</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -103). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -6073,32 +6073,32 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -9.5</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5226</v>
+        <v>0.4968</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-109</v>
+        <v>101</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-104</v>
+        <v>113</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 52.3% (fair -109). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -6139,32 +6139,32 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun +5.5</t>
+          <t>Chicago Sky</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5201</v>
+        <v>0.5561</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-108</v>
+        <v>-125</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-104</v>
+        <v>-113</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -6197,9 +6197,339 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>23:05</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>0.5033</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>-101</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I23" s="13">
+        <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
+        <v/>
+      </c>
+      <c r="J23" s="16">
+        <f>IF($H$23="","",$F$23*IF($H$23&lt;0,-100/$H$23,$H$23/100)-(1-$F$23))</f>
+        <v/>
+      </c>
+      <c r="K23" s="17">
+        <f>IF($H$23="","",MAX(0,($F$23*IF($H$23&lt;0,-100/$H$23,$H$23/100)-(1-$F$23))/IF($H$23&lt;0,-100/$H$23,$H$23/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L23" s="18">
+        <f>IF($H$23="","",ROUND(MIN($K$23,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M23" s="12">
+        <f>IF($J$23="","",IF($J$23&lt;0,"Pass",IF($J$23&lt;'Settings'!$B$4,"Thin",IF($J$23&lt;0.06,"✅ Sharp band",IF($J$23&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N23" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.3% (fair -101). Your call.</t>
+        </is>
+      </c>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="16">
+        <f>IF(OR($H$23="",$O$23=""),"",(1+IF($H$23&lt;0,-100/$H$23,$H$23/100))/(1+IF($O$23&lt;0,-100/$O$23,$O$23/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.4067</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>146</v>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v>156</v>
+      </c>
+      <c r="I24" s="13">
+        <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
+        <v/>
+      </c>
+      <c r="J24" s="16">
+        <f>IF($H$24="","",$F$24*IF($H$24&lt;0,-100/$H$24,$H$24/100)-(1-$F$24))</f>
+        <v/>
+      </c>
+      <c r="K24" s="17">
+        <f>IF($H$24="","",MAX(0,($F$24*IF($H$24&lt;0,-100/$H$24,$H$24/100)-(1-$F$24))/IF($H$24&lt;0,-100/$H$24,$H$24/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L24" s="18">
+        <f>IF($H$24="","",ROUND(MIN($K$24,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M24" s="12">
+        <f>IF($J$24="","",IF($J$24&lt;0,"Pass",IF($J$24&lt;'Settings'!$B$4,"Thin",IF($J$24&lt;0.06,"✅ Sharp band",IF($J$24&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N24" s="19" t="inlineStr">
+        <is>
+          <t>Model 40.7% (fair +146). Your call.</t>
+        </is>
+      </c>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="16">
+        <f>IF(OR($H$24="",$O$24=""),"",(1+IF($H$24&lt;0,-100/$H$24,$H$24/100))/(1+IF($O$24&lt;0,-100/$O$24,$O$24/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>New York Mets @ Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>23:10</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Over 9.5</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>0.5187</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>-108</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="I25" s="13">
+        <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
+        <v/>
+      </c>
+      <c r="J25" s="16">
+        <f>IF($H$25="","",$F$25*IF($H$25&lt;0,-100/$H$25,$H$25/100)-(1-$F$25))</f>
+        <v/>
+      </c>
+      <c r="K25" s="17">
+        <f>IF($H$25="","",MAX(0,($F$25*IF($H$25&lt;0,-100/$H$25,$H$25/100)-(1-$F$25))/IF($H$25&lt;0,-100/$H$25,$H$25/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>IF($H$25="","",ROUND(MIN($K$25,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M25" s="12">
+        <f>IF($J$25="","",IF($J$25&lt;0,"Pass",IF($J$25&lt;'Settings'!$B$4,"Thin",IF($J$25&lt;0.06,"✅ Sharp band",IF($J$25&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N25" s="19" t="inlineStr">
+        <is>
+          <t>Model 51.9% (fair -108). Your call.</t>
+        </is>
+      </c>
+      <c r="O25" s="15" t="n"/>
+      <c r="P25" s="16">
+        <f>IF(OR($H$25="",$O$25=""),"",(1+IF($H$25&lt;0,-100/$H$25,$H$25/100))/(1+IF($O$25&lt;0,-100/$O$25,$O$25/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Storm @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Indiana Fever -10.5</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.4947</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I26" s="13">
+        <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
+        <v/>
+      </c>
+      <c r="J26" s="16">
+        <f>IF($H$26="","",$F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))</f>
+        <v/>
+      </c>
+      <c r="K26" s="17">
+        <f>IF($H$26="","",MAX(0,($F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))/IF($H$26&lt;0,-100/$H$26,$H$26/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
+        <f>IF($H$26="","",ROUND(MIN($K$26,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M26" s="12">
+        <f>IF($J$26="","",IF($J$26&lt;0,"Pass",IF($J$26&lt;'Settings'!$B$4,"Thin",IF($J$26&lt;0.06,"✅ Sharp band",IF($J$26&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.5% (fair +102). Your call.</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="16">
+        <f>IF(OR($H$26="",$O$26=""),"",(1+IF($H$26&lt;0,-100/$H$26,$H$26/100))/(1+IF($O$26&lt;0,-100/$O$26,$O$26/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Atlanta Dream @ Toronto Tempo</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Over 183.5</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0.5012</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>-100</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v>104</v>
+      </c>
+      <c r="I27" s="13">
+        <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
+        <v/>
+      </c>
+      <c r="J27" s="16">
+        <f>IF($H$27="","",$F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))</f>
+        <v/>
+      </c>
+      <c r="K27" s="17">
+        <f>IF($H$27="","",MAX(0,($F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))/IF($H$27&lt;0,-100/$H$27,$H$27/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
+        <f>IF($H$27="","",ROUND(MIN($K$27,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M27" s="12">
+        <f>IF($J$27="","",IF($J$27&lt;0,"Pass",IF($J$27&lt;'Settings'!$B$4,"Thin",IF($J$27&lt;0.06,"✅ Sharp band",IF($J$27&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N27" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.1% (fair -100). Your call.</t>
+        </is>
+      </c>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="16">
+        <f>IF(OR($H$27="",$O$27=""),"",(1+IF($H$27&lt;0,-100/$H$27,$H$27/100))/(1+IF($O$27&lt;0,-100/$O$27,$O$27/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J22">
+  <conditionalFormatting sqref="J5:J27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -6221,7 +6551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P56"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6365,13 +6695,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4516</v>
+        <v>0.452</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>121</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -6431,7 +6761,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5484</v>
+        <v>0.548</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-121</v>
@@ -6497,10 +6827,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5067</v>
+        <v>0.5187</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-103</v>
+        <v>-108</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -6527,7 +6857,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -6563,13 +6893,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4933</v>
+        <v>0.4813</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -6593,7 +6923,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -6629,13 +6959,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3632</v>
+        <v>0.3771</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -6659,7 +6989,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 36.3% (fair +175). Your call.</t>
+          <t>Model 37.7% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -6695,13 +7025,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6368</v>
+        <v>0.6229</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-175</v>
+        <v>-165</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>158</v>
+        <v>-163</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -6725,7 +7055,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 63.7% (fair -175). Your call.</t>
+          <t>Model 62.3% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -6761,10 +7091,10 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4269944000000001</v>
+        <v>0.4250646</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>127</v>
@@ -6791,7 +7121,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 42.7% (fair +134). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -6827,10 +7157,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5730055999999999</v>
+        <v>0.5749354</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-134</v>
+        <v>-135</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>122</v>
@@ -6857,7 +7187,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -6893,10 +7223,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.649</v>
+        <v>0.6299</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-185</v>
+        <v>-170</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>100</v>
@@ -6923,7 +7253,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 64.9% (fair -185). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -6959,10 +7289,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.351</v>
+        <v>0.3701</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>144</v>
@@ -6989,7 +7319,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 35.1% (fair +185). Your call.</t>
+          <t>Model 37.0% (fair +170). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -7025,13 +7355,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.3865</v>
+        <v>0.3888</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -7055,7 +7385,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 38.6% (fair +159). Your call.</t>
+          <t>Model 38.9% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -7091,10 +7421,10 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6134999999999999</v>
+        <v>0.6112</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-159</v>
+        <v>-157</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>-163</v>
@@ -7121,7 +7451,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 61.3% (fair -159). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -7157,10 +7487,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4249418</v>
+        <v>0.4230384</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>127</v>
@@ -7187,7 +7517,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -7223,10 +7553,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5750582</v>
+        <v>0.5769616</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-135</v>
+        <v>-136</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>122</v>
@@ -7253,7 +7583,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 57.5% (fair -135). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -7289,10 +7619,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6535</v>
+        <v>0.6559</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-189</v>
+        <v>-191</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>100</v>
@@ -7319,7 +7649,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 65.3% (fair -189). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -7355,10 +7685,10 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3465</v>
+        <v>0.3441</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>144</v>
@@ -7385,7 +7715,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 34.7% (fair +189). Your call.</t>
+          <t>Model 34.4% (fair +191). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -7421,13 +7751,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.3851</v>
+        <v>0.3905</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -7451,7 +7781,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 38.5% (fair +160). Your call.</t>
+          <t>Model 39.1% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -7487,10 +7817,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.6149</v>
+        <v>0.6094999999999999</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-160</v>
+        <v>-156</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>-163</v>
@@ -7517,7 +7847,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 61.5% (fair -160). Your call.</t>
+          <t>Model 60.9% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -7553,10 +7883,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4936</v>
+        <v>0.4967</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>-108</v>
@@ -7583,7 +7913,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +103). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -7619,13 +7949,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5064</v>
+        <v>0.5033</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-103</v>
+        <v>-101</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -7649,7 +7979,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -103). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -7685,13 +8015,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4733000000000001</v>
+        <v>0.4587</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -7715,7 +8045,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +111). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -7751,13 +8081,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5266999999999999</v>
+        <v>0.5413</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-111</v>
+        <v>-118</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-108</v>
+        <v>-117</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -7781,7 +8111,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -111). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -7798,32 +8128,32 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4099</v>
+        <v>0.5503</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>144</v>
+        <v>-122</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>138</v>
+        <v>-108</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -7847,7 +8177,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 41.0% (fair +144). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -7864,32 +8194,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Under 7.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5901</v>
+        <v>0.4497</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-144</v>
+        <v>122</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-144</v>
+        <v>100</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -7913,7 +8243,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -7930,32 +8260,32 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Cleveland Guardians -1.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4526</v>
+        <v>0.3426</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>121</v>
+        <v>192</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>122</v>
+        <v>175</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -7979,7 +8309,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 34.3% (fair +192). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -7996,32 +8326,32 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates +1.5</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5474</v>
+        <v>0.6574</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-121</v>
+        <v>-192</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-117</v>
+        <v>178</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -8045,7 +8375,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 65.7% (fair -192). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -8062,7 +8392,7 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -8072,22 +8402,22 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.6086</v>
+        <v>0.4091</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-155</v>
+        <v>144</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -8111,7 +8441,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -155). Your call.</t>
+          <t>Model 40.9% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -8128,7 +8458,7 @@
       </c>
       <c r="B32" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C32" s="20" t="inlineStr">
@@ -8138,22 +8468,22 @@
       </c>
       <c r="D32" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.3914</v>
+        <v>0.5909</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>155</v>
+        <v>-144</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>144</v>
+        <v>-144</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -8177,7 +8507,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +155). Your call.</t>
+          <t>Model 59.1% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -8204,22 +8534,22 @@
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays -1.5</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.368</v>
+        <v>0.4487</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>172</v>
+        <v>123</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>175</v>
+        <v>122</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -8243,7 +8573,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 36.8% (fair +172). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -8270,22 +8600,22 @@
       </c>
       <c r="D34" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E34" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox +1.5</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.632</v>
+        <v>0.5513</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-172</v>
+        <v>-123</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>160</v>
+        <v>-122</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -8309,7 +8639,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 63.2% (fair -172). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -8326,32 +8656,32 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4001</v>
+        <v>0.598</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>150</v>
+        <v>-149</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>163</v>
+        <v>100</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -8375,7 +8705,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 40.0% (fair +150). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -8392,32 +8722,32 @@
       </c>
       <c r="B36" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C36" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D36" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E36" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Under 7.5</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5999</v>
+        <v>0.402</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-150</v>
+        <v>149</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>-170</v>
+        <v>144</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -8441,7 +8771,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 60.0% (fair -150). Your call.</t>
+          <t>Model 40.2% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -8458,32 +8788,32 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Toronto Blue Jays -1.5</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4379999999999999</v>
+        <v>0.3698</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>128</v>
+        <v>170</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -8507,7 +8837,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 43.8% (fair +128). Your call.</t>
+          <t>Model 37.0% (fair +170). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -8524,32 +8854,32 @@
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D38" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E38" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Chicago White Sox +1.5</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.6302</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-128</v>
+        <v>-170</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>-127</v>
+        <v>178</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -8573,7 +8903,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -8590,12 +8920,12 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -8605,17 +8935,17 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.5064</v>
+        <v>0.4067</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-103</v>
+        <v>146</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>-117</v>
+        <v>156</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -8639,7 +8969,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -103). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -8656,12 +8986,12 @@
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D40" s="20" t="inlineStr">
@@ -8671,17 +9001,17 @@
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4936</v>
+        <v>0.5933</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>103</v>
+        <v>-146</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>113</v>
+        <v>-163</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -8705,7 +9035,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +103). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -8722,12 +9052,12 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
@@ -8737,17 +9067,17 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.4826</v>
+        <v>0.4439</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -8771,7 +9101,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -8788,12 +9118,12 @@
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C42" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D42" s="20" t="inlineStr">
@@ -8803,17 +9133,17 @@
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5174</v>
+        <v>0.5561</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-107</v>
+        <v>-125</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-113</v>
+        <v>-127</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -8837,7 +9167,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -8854,7 +9184,7 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
@@ -8864,22 +9194,22 @@
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.5431</v>
+        <v>0.5032</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>-119</v>
+        <v>-101</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>-125</v>
+        <v>-113</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -8903,7 +9233,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -8920,7 +9250,7 @@
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr">
@@ -8930,22 +9260,22 @@
       </c>
       <c r="D44" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4569</v>
+        <v>0.4968</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -8969,7 +9299,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -8996,22 +9326,22 @@
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals +1.5</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.5931999999999999</v>
+        <v>0.4922</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>-146</v>
+        <v>103</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>-165</v>
+        <v>104</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -9035,7 +9365,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 59.3% (fair -146). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -9062,22 +9392,22 @@
       </c>
       <c r="D46" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E46" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres -1.5</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4068000000000001</v>
+        <v>0.5078</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>146</v>
+        <v>-103</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>140</v>
+        <v>-104</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -9101,7 +9431,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 40.7% (fair +146). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -9118,31 +9448,33 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.3456</v>
+        <v>0.3923</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>189</v>
-      </c>
-      <c r="H47" s="15" t="n"/>
+        <v>155</v>
+      </c>
+      <c r="H47" s="15" t="n">
+        <v>108</v>
+      </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
         <v/>
@@ -9165,7 +9497,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 34.6% (fair +189). Your call.</t>
+          <t>Model 39.2% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -9182,31 +9514,33 @@
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D48" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E48" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.6544</v>
+        <v>0.6077</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-189</v>
-      </c>
-      <c r="H48" s="15" t="n"/>
+        <v>-155</v>
+      </c>
+      <c r="H48" s="15" t="n">
+        <v>105</v>
+      </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
         <v/>
@@ -9229,7 +9563,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 65.4% (fair -189). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -9246,31 +9580,33 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ Los Angeles Angels</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Kansas City Royals +1.5</t>
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.5383</v>
+        <v>0.5988</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>-117</v>
-      </c>
-      <c r="H49" s="15" t="n"/>
+        <v>-149</v>
+      </c>
+      <c r="H49" s="15" t="n">
+        <v>-163</v>
+      </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
         <v/>
@@ -9293,7 +9629,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -117). Your call.</t>
+          <t>Model 59.9% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -9310,31 +9646,33 @@
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ Los Angeles Angels</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D50" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>San Diego Padres -1.5</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4617</v>
+        <v>0.4012</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>117</v>
-      </c>
-      <c r="H50" s="15" t="n"/>
+        <v>149</v>
+      </c>
+      <c r="H50" s="15" t="n">
+        <v>150</v>
+      </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
         <v/>
@@ -9357,7 +9695,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +117). Your call.</t>
+          <t>Model 40.1% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -9374,12 +9712,12 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Athletics</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
@@ -9389,14 +9727,14 @@
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.4984</v>
+        <v>0.3456</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13">
@@ -9421,7 +9759,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 34.6% (fair +189). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -9438,12 +9776,12 @@
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Athletics</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D52" s="20" t="inlineStr">
@@ -9453,14 +9791,14 @@
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.5016</v>
+        <v>0.6544</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>-101</v>
+        <v>-189</v>
       </c>
       <c r="H52" s="15" t="n"/>
       <c r="I52" s="13">
@@ -9485,7 +9823,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 65.4% (fair -189). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -9502,12 +9840,12 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Detroit Tigers @ Los Angeles Angels</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>01:38</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
@@ -9517,14 +9855,14 @@
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.4814</v>
+        <v>0.5327</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>108</v>
+        <v>-114</v>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13">
@@ -9549,7 +9887,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -9566,12 +9904,12 @@
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Detroit Tigers @ Los Angeles Angels</t>
         </is>
       </c>
       <c r="C54" s="20" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>01:38</t>
         </is>
       </c>
       <c r="D54" s="20" t="inlineStr">
@@ -9581,14 +9919,14 @@
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.5185999999999999</v>
+        <v>0.4673</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-108</v>
+        <v>114</v>
       </c>
       <c r="H54" s="15" t="n"/>
       <c r="I54" s="13">
@@ -9613,7 +9951,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -9630,12 +9968,12 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Washington Nationals @ Athletics</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
@@ -9645,14 +9983,14 @@
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.5019</v>
+        <v>0.5006</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>-101</v>
+        <v>-100</v>
       </c>
       <c r="H55" s="15" t="n"/>
       <c r="I55" s="13">
@@ -9677,7 +10015,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -9694,12 +10032,12 @@
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Washington Nationals @ Athletics</t>
         </is>
       </c>
       <c r="C56" s="20" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="D56" s="20" t="inlineStr">
@@ -9709,14 +10047,14 @@
       </c>
       <c r="E56" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4981</v>
+        <v>0.4995</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H56" s="15" t="n"/>
       <c r="I56" s="13">
@@ -9741,7 +10079,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 50.0% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -9750,9 +10088,265 @@
         <v/>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="F57" s="13" t="n">
+        <v>0.4814</v>
+      </c>
+      <c r="G57" s="14" t="n">
+        <v>108</v>
+      </c>
+      <c r="H57" s="15" t="n"/>
+      <c r="I57" s="13">
+        <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
+        <v/>
+      </c>
+      <c r="J57" s="16">
+        <f>IF($H$57="","",$F$57*IF($H$57&lt;0,-100/$H$57,$H$57/100)-(1-$F$57))</f>
+        <v/>
+      </c>
+      <c r="K57" s="17">
+        <f>IF($H$57="","",MAX(0,($F$57*IF($H$57&lt;0,-100/$H$57,$H$57/100)-(1-$F$57))/IF($H$57&lt;0,-100/$H$57,$H$57/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L57" s="18">
+        <f>IF($H$57="","",ROUND(MIN($K$57,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M57" s="12">
+        <f>IF($J$57="","",IF($J$57&lt;0,"Pass",IF($J$57&lt;'Settings'!$B$4,"Thin",IF($J$57&lt;0.06,"✅ Sharp band",IF($J$57&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N57" s="19" t="inlineStr">
+        <is>
+          <t>Model 48.1% (fair +108). Your call.</t>
+        </is>
+      </c>
+      <c r="O57" s="15" t="n"/>
+      <c r="P57" s="16">
+        <f>IF(OR($H$57="",$O$57=""),"",(1+IF($H$57&lt;0,-100/$H$57,$H$57/100))/(1+IF($O$57&lt;0,-100/$O$57,$O$57/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B58" s="20" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>0.5185999999999999</v>
+      </c>
+      <c r="G58" s="14" t="n">
+        <v>-108</v>
+      </c>
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="13">
+        <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
+        <v/>
+      </c>
+      <c r="J58" s="16">
+        <f>IF($H$58="","",$F$58*IF($H$58&lt;0,-100/$H$58,$H$58/100)-(1-$F$58))</f>
+        <v/>
+      </c>
+      <c r="K58" s="17">
+        <f>IF($H$58="","",MAX(0,($F$58*IF($H$58&lt;0,-100/$H$58,$H$58/100)-(1-$F$58))/IF($H$58&lt;0,-100/$H$58,$H$58/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L58" s="18">
+        <f>IF($H$58="","",ROUND(MIN($K$58,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M58" s="12">
+        <f>IF($J$58="","",IF($J$58&lt;0,"Pass",IF($J$58&lt;'Settings'!$B$4,"Thin",IF($J$58&lt;0.06,"✅ Sharp band",IF($J$58&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N58" s="19" t="inlineStr">
+        <is>
+          <t>Model 51.9% (fair -108). Your call.</t>
+        </is>
+      </c>
+      <c r="O58" s="15" t="n"/>
+      <c r="P58" s="16">
+        <f>IF(OR($H$58="",$O$58=""),"",(1+IF($H$58&lt;0,-100/$H$58,$H$58/100))/(1+IF($O$58&lt;0,-100/$O$58,$O$58/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants @ Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E59" s="12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="F59" s="13" t="n">
+        <v>0.4992</v>
+      </c>
+      <c r="G59" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H59" s="15" t="n"/>
+      <c r="I59" s="13">
+        <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
+        <v/>
+      </c>
+      <c r="J59" s="16">
+        <f>IF($H$59="","",$F$59*IF($H$59&lt;0,-100/$H$59,$H$59/100)-(1-$F$59))</f>
+        <v/>
+      </c>
+      <c r="K59" s="17">
+        <f>IF($H$59="","",MAX(0,($F$59*IF($H$59&lt;0,-100/$H$59,$H$59/100)-(1-$F$59))/IF($H$59&lt;0,-100/$H$59,$H$59/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L59" s="18">
+        <f>IF($H$59="","",ROUND(MIN($K$59,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M59" s="12">
+        <f>IF($J$59="","",IF($J$59&lt;0,"Pass",IF($J$59&lt;'Settings'!$B$4,"Thin",IF($J$59&lt;0.06,"✅ Sharp band",IF($J$59&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N59" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.9% (fair +100). Your call.</t>
+        </is>
+      </c>
+      <c r="O59" s="15" t="n"/>
+      <c r="P59" s="16">
+        <f>IF(OR($H$59="",$O$59=""),"",(1+IF($H$59&lt;0,-100/$H$59,$H$59/100))/(1+IF($O$59&lt;0,-100/$O$59,$O$59/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B60" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco Giants @ Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.5008</v>
+      </c>
+      <c r="G60" s="14" t="n">
+        <v>-100</v>
+      </c>
+      <c r="H60" s="15" t="n"/>
+      <c r="I60" s="13">
+        <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
+        <v/>
+      </c>
+      <c r="J60" s="16">
+        <f>IF($H$60="","",$F$60*IF($H$60&lt;0,-100/$H$60,$H$60/100)-(1-$F$60))</f>
+        <v/>
+      </c>
+      <c r="K60" s="17">
+        <f>IF($H$60="","",MAX(0,($F$60*IF($H$60&lt;0,-100/$H$60,$H$60/100)-(1-$F$60))/IF($H$60&lt;0,-100/$H$60,$H$60/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L60" s="18">
+        <f>IF($H$60="","",ROUND(MIN($K$60,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M60" s="12">
+        <f>IF($J$60="","",IF($J$60&lt;0,"Pass",IF($J$60&lt;'Settings'!$B$4,"Thin",IF($J$60&lt;0.06,"✅ Sharp band",IF($J$60&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N60" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.1% (fair -100). Your call.</t>
+        </is>
+      </c>
+      <c r="O60" s="15" t="n"/>
+      <c r="P60" s="16">
+        <f>IF(OR($H$60="",$O$60=""),"",(1+IF($H$60&lt;0,-100/$H$60,$H$60/100))/(1+IF($O$60&lt;0,-100/$O$60,$O$60/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J56">
+  <conditionalFormatting sqref="J5:J60">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -9924,7 +10518,7 @@
         <v>220</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -10050,7 +10644,7 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6058</v>
+        <v>0.6064000000000001</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>-154</v>
@@ -10116,13 +10710,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3942</v>
+        <v>0.3935999999999999</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>154</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -10182,10 +10776,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4956023001506284</v>
+        <v>0.499</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>100</v>
@@ -10212,7 +10806,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10248,13 +10842,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5043976998493716</v>
+        <v>0.501</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-102</v>
+        <v>-100</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -10278,7 +10872,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -10314,13 +10908,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4347</v>
+        <v>0.4286</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -10344,7 +10938,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10380,13 +10974,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5653</v>
+        <v>0.5714</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-130</v>
+        <v>-133</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -10410,7 +11004,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10442,14 +11036,14 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 176.5</t>
+          <t>Over 177.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5405282796034565</v>
+        <v>0.5086000000000001</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-118</v>
+        <v>-104</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>100</v>
@@ -10476,7 +11070,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -10508,17 +11102,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 176.5</t>
+          <t>Under 177.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4594717203965435</v>
+        <v>0.4913999999999999</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -10542,7 +11136,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10574,17 +11168,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings -2</t>
+          <t>Dallas Wings -2.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.56287707702024</v>
+        <v>0.5473217733731714</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-129</v>
+        <v>-121</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -10608,7 +11202,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 54.7% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -10640,14 +11234,14 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty +2</t>
+          <t>New York Liberty +2.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4061229229797599</v>
+        <v>0.4526782266268286</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>122</v>
@@ -10674,7 +11268,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 40.6% (fair +146). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -10842,10 +11436,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5702</v>
+        <v>0.6676848981971866</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-133</v>
+        <v>-201</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>113</v>
@@ -10872,7 +11466,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -133). Your call.</t>
+          <t>Model 66.8% (fair -201). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -10908,13 +11502,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4298</v>
+        <v>0.3323151018028134</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>133</v>
+        <v>201</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-110</v>
+        <v>108</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -10938,7 +11532,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 43.0% (fair +133). Your call.</t>
+          <t>Model 33.2% (fair +201). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -10970,17 +11564,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -9.5</t>
+          <t>Indiana Fever -10.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5226</v>
+        <v>0.4947</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-109</v>
+        <v>102</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -11004,7 +11598,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 52.3% (fair -109). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11036,17 +11630,17 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm +9.5</t>
+          <t>Seattle Storm +10.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4774</v>
+        <v>0.5053000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>109</v>
+        <v>-102</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -11070,7 +11664,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 47.7% (fair +109). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -11178,7 +11772,7 @@
         <v>209</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -11234,17 +11828,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 181.5</t>
+          <t>Over 183.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.53</v>
+        <v>0.5012</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-113</v>
+        <v>-100</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-105</v>
+        <v>104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -11268,7 +11862,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -11300,14 +11894,14 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 181.5</t>
+          <t>Under 183.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.47</v>
+        <v>0.4988</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>-105</v>
@@ -11334,7 +11928,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -11366,17 +11960,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +7.5</t>
+          <t>Toronto Tempo +6.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5643</v>
+        <v>0.542</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-130</v>
+        <v>-118</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -11400,7 +11994,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -130). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -11432,14 +12026,14 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream -7.5</t>
+          <t>Atlanta Dream -6.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4357</v>
+        <v>0.458</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>-105</v>
@@ -11466,7 +12060,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 43.6% (fair +130). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -11502,13 +12096,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4389</v>
+        <v>0.4439</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11532,7 +12126,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 43.9% (fair +128). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -11568,13 +12162,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5611</v>
+        <v>0.5561</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-128</v>
+        <v>-125</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -11598,7 +12192,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -11634,10 +12228,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5399</v>
+        <v>0.5482</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-117</v>
+        <v>-121</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>-105</v>
@@ -11664,7 +12258,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -11700,13 +12294,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4601</v>
+        <v>0.4518</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>-110</v>
+        <v>104</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11730,7 +12324,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -11766,10 +12360,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5053</v>
+        <v>0.5036</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-102</v>
+        <v>-101</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>-108</v>
@@ -11796,7 +12390,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 50.4% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -11832,13 +12426,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4947</v>
+        <v>0.4964</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-105</v>
+        <v>-108</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -11862,7 +12456,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 49.6% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -11904,7 +12498,7 @@
         <v>150</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -12030,13 +12624,13 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.5842000000000001</v>
+        <v>0.5848</v>
       </c>
       <c r="G37" s="14" t="n">
         <v>-141</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -12060,7 +12654,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 58.4% (fair -141). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -12096,7 +12690,7 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4157999999999999</v>
+        <v>0.4152</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>141</v>
@@ -12126,7 +12720,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 41.6% (fair +141). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -12162,13 +12756,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.4799</v>
+        <v>0.4866</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -12192,7 +12786,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 48.7% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12228,13 +12822,13 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5201</v>
+        <v>0.5134000000000001</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>-108</v>
+        <v>-106</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -12258,7 +12852,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 51.3% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -12441,7 +13035,7 @@
         <v>243</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>275</v>
+        <v>205</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -12507,7 +13101,7 @@
         <v>130</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -12573,7 +13167,7 @@
         <v>243</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -12639,7 +13233,7 @@
         <v>130</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -12705,7 +13299,7 @@
         <v>243</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>575</v>
+        <v>585</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -12771,7 +13365,7 @@
         <v>130</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-218</v>
+        <v>-220</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>

</xml_diff>

<commit_message>
data: hourly update 2026-07-16 19:25Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-16.xlsx
+++ b/data/output/workbook/2026-07-16.xlsx
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 14:12</t>
+          <t>2026-07-16 15:25</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5017,12 +5017,12 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -5032,17 +5032,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates +1.5</t>
+          <t>Miami Marlins +1.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6574</v>
+        <v>0.6105</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-192</v>
+        <v>-157</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>178</v>
+        <v>213</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 65.7% (fair -192). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5083,12 +5083,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -5098,14 +5098,14 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox +1.5</t>
+          <t>Pittsburgh Pirates +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6302</v>
+        <v>0.6574</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-170</v>
+        <v>-192</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>178</v>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 63.0% (fair -170). Your call.</t>
+          <t>Model 65.7% (fair -192). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5149,32 +5149,32 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Chicago White Sox +1.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6559</v>
+        <v>0.6302</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-191</v>
+        <v>-170</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>100</v>
+        <v>178</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 65.6% (fair -191). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5220,27 +5220,27 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Tampa Bay Rays +1.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.6006</v>
+        <v>0.6094999999999999</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-150</v>
+        <v>-156</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>100</v>
+        <v>156</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 60.1% (fair -150). Your call.</t>
+          <t>Model 60.9% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5281,32 +5281,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Tampa Bay Rays +1.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.598</v>
+        <v>0.5847</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-149</v>
+        <v>-141</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>100</v>
+        <v>156</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 59.8% (fair -149). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -5347,32 +5347,32 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Colorado Rockies -1.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5729</v>
+        <v>0.5564</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-134</v>
+        <v>-125</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -5413,12 +5413,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -5428,14 +5428,14 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5814</v>
+        <v>0.6559</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-139</v>
+        <v>-191</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>100</v>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 58.1% (fair -139). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -5489,22 +5489,22 @@
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4113</v>
+        <v>0.6264999999999999</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>143</v>
+        <v>-168</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>178</v>
+        <v>100</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 41.1% (fair +143). Your call.</t>
+          <t>Model 62.6% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -5545,12 +5545,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -5560,17 +5560,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5848</v>
+        <v>0.6077</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-141</v>
+        <v>-155</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-106</v>
+        <v>106</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -5611,12 +5611,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -5626,17 +5626,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5503</v>
+        <v>0.598</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-122</v>
+        <v>-149</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -5677,32 +5677,32 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +6.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.542</v>
+        <v>0.5729</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-118</v>
+        <v>-134</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 57.3% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -5743,32 +5743,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.3905</v>
+        <v>0.5503</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>156</v>
+        <v>-122</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>178</v>
+        <v>113</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -5809,32 +5809,32 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5473</v>
+        <v>0.4153</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-121</v>
+        <v>141</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>-104</v>
+        <v>178</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -5885,22 +5885,22 @@
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun +5.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5145999999999999</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="G18" s="14" t="n">
+        <v>-142</v>
+      </c>
+      <c r="H18" s="15" t="n">
         <v>-106</v>
-      </c>
-      <c r="H18" s="15" t="n">
-        <v>108</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Atlanta Dream @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -5951,22 +5951,22 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Toronto Tempo +6.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5482</v>
+        <v>0.5426</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-121</v>
+        <v>-119</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-105</v>
+        <v>108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -6022,17 +6022,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies +1.5</t>
+          <t>Cincinnati Reds +1.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.6559</v>
+        <v>0.4436</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-191</v>
+        <v>125</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-165</v>
+        <v>150</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 65.6% (fair -191). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -6073,32 +6073,32 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Seattle Storm @ Indiana Fever</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Over 175.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5041</v>
+        <v>0.5692</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-102</v>
+        <v>-132</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>108</v>
+        <v>-108</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 56.9% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -6139,32 +6139,32 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5561</v>
+        <v>0.5442</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-125</v>
+        <v>-119</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-113</v>
+        <v>100</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -6205,32 +6205,32 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5337000000000001</v>
+        <v>0.3905</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-114</v>
+        <v>156</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-104</v>
+        <v>178</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -6254,7 +6254,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -114). Your call.</t>
+          <t>Model 39.1% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -6271,12 +6271,12 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -6286,17 +6286,17 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Chicago Sky</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5026</v>
+        <v>0.5534</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-101</v>
+        <v>-124</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>108</v>
+        <v>-108</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -6337,32 +6337,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Connecticut Sun +5.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4032</v>
+        <v>0.517</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>148</v>
+        <v>-107</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 40.3% (fair +148). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -6403,32 +6403,32 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Over 185.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.6041</v>
+        <v>0.5147</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-153</v>
+        <v>-106</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-144</v>
+        <v>104</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 60.4% (fair -153). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -6469,32 +6469,32 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5012</v>
+        <v>0.5041</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-100</v>
+        <v>-102</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -6527,9 +6527,141 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>23:05</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.5026</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>-101</v>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I28" s="13">
+        <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
+        <v/>
+      </c>
+      <c r="J28" s="16">
+        <f>IF($H$28="","",$F$28*IF($H$28&lt;0,-100/$H$28,$H$28/100)-(1-$F$28))</f>
+        <v/>
+      </c>
+      <c r="K28" s="17">
+        <f>IF($H$28="","",MAX(0,($F$28*IF($H$28&lt;0,-100/$H$28,$H$28/100)-(1-$F$28))/IF($H$28&lt;0,-100/$H$28,$H$28/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
+        <f>IF($H$28="","",ROUND(MIN($K$28,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M28" s="12">
+        <f>IF($J$28="","",IF($J$28&lt;0,"Pass",IF($J$28&lt;'Settings'!$B$4,"Thin",IF($J$28&lt;0.06,"✅ Sharp band",IF($J$28&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N28" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.3% (fair -101). Your call.</t>
+        </is>
+      </c>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="16">
+        <f>IF(OR($H$28="",$O$28=""),"",(1+IF($H$28&lt;0,-100/$H$28,$H$28/100))/(1+IF($O$28&lt;0,-100/$O$28,$O$28/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Under 8.5</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0.5211</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>-109</v>
+      </c>
+      <c r="H29" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="I29" s="13">
+        <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
+        <v/>
+      </c>
+      <c r="J29" s="16">
+        <f>IF($H$29="","",$F$29*IF($H$29&lt;0,-100/$H$29,$H$29/100)-(1-$F$29))</f>
+        <v/>
+      </c>
+      <c r="K29" s="17">
+        <f>IF($H$29="","",MAX(0,($F$29*IF($H$29&lt;0,-100/$H$29,$H$29/100)-(1-$F$29))/IF($H$29&lt;0,-100/$H$29,$H$29/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L29" s="18">
+        <f>IF($H$29="","",ROUND(MIN($K$29,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M29" s="12">
+        <f>IF($J$29="","",IF($J$29&lt;0,"Pass",IF($J$29&lt;'Settings'!$B$4,"Thin",IF($J$29&lt;0.06,"✅ Sharp band",IF($J$29&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N29" s="19" t="inlineStr">
+        <is>
+          <t>Model 52.1% (fair -109). Your call.</t>
+        </is>
+      </c>
+      <c r="O29" s="15" t="n"/>
+      <c r="P29" s="16">
+        <f>IF(OR($H$29="",$O$29=""),"",(1+IF($H$29&lt;0,-100/$H$29,$H$29/100))/(1+IF($O$29&lt;0,-100/$O$29,$O$29/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J27">
+  <conditionalFormatting sqref="J5:J29">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -6551,7 +6683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6695,7 +6827,7 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4545</v>
+        <v>0.4547</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>120</v>
@@ -6761,13 +6893,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5455</v>
+        <v>0.5453</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-120</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-119</v>
+        <v>-120</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -6827,10 +6959,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4425</v>
+        <v>0.4281</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>117</v>
@@ -6857,7 +6989,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 42.8% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -6893,13 +7025,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4751</v>
+        <v>0.4899000000000001</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -6923,7 +7055,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -6959,13 +7091,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3754</v>
+        <v>0.3735</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -6989,7 +7121,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 37.5% (fair +166). Your call.</t>
+          <t>Model 37.4% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -7025,10 +7157,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6246</v>
+        <v>0.6265000000000001</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-166</v>
+        <v>-168</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>-163</v>
@@ -7055,7 +7187,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 62.5% (fair -166). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -7223,10 +7355,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.6006</v>
+        <v>0.6264999999999999</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-150</v>
+        <v>-168</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>100</v>
@@ -7253,7 +7385,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 60.1% (fair -150). Your call.</t>
+          <t>Model 62.6% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -7289,10 +7421,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3994</v>
+        <v>0.3735000000000001</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>144</v>
@@ -7319,7 +7451,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +150). Your call.</t>
+          <t>Model 37.4% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -7355,10 +7487,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4113</v>
+        <v>0.4153</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>178</v>
@@ -7385,7 +7517,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 41.1% (fair +143). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -7421,13 +7553,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5887</v>
+        <v>0.5847</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-143</v>
+        <v>-141</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-163</v>
+        <v>156</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -7451,7 +7583,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -7823,7 +7955,7 @@
         <v>-156</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-163</v>
+        <v>156</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -8021,7 +8153,7 @@
         <v>134</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -8087,7 +8219,7 @@
         <v>-134</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -8279,13 +8411,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4587</v>
+        <v>0.4617</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -8309,7 +8441,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 46.2% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -8345,10 +8477,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5413</v>
+        <v>0.5383</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-118</v>
+        <v>-117</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-117</v>
@@ -8375,7 +8507,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 53.8% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -8411,13 +8543,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5473</v>
+        <v>0.5442</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-121</v>
+        <v>-119</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -8441,7 +8573,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -8477,10 +8609,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4527</v>
+        <v>0.4558</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -8507,7 +8639,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -8675,13 +8807,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.3959</v>
+        <v>0.3587399999999999</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>138</v>
+        <v>186</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -8705,7 +8837,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 39.6% (fair +153). Your call.</t>
+          <t>Model 35.9% (fair +179). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -8741,13 +8873,13 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.6041</v>
+        <v>0.6412600000000001</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-153</v>
+        <v>-179</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>-144</v>
+        <v>-105</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -8771,7 +8903,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 60.4% (fair -153). Your call.</t>
+          <t>Model 64.1% (fair -179). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -8788,7 +8920,7 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
@@ -8798,22 +8930,22 @@
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4518</v>
+        <v>0.4909</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>122</v>
+        <v>-104</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -8837,7 +8969,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -8854,7 +8986,7 @@
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr">
@@ -8864,22 +8996,22 @@
       </c>
       <c r="D38" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E38" s="20" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5482</v>
+        <v>0.5091</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-121</v>
+        <v>-104</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>-117</v>
+        <v>-105</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -8903,7 +9035,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -8920,7 +9052,7 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
@@ -8930,22 +9062,22 @@
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Atlanta Braves -1.5</t>
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.598</v>
+        <v>0.4601</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-149</v>
+        <v>117</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -8969,7 +9101,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 59.8% (fair -149). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -8986,7 +9118,7 @@
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr">
@@ -8996,22 +9128,22 @@
       </c>
       <c r="D40" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Texas Rangers +1.5</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.402</v>
+        <v>0.5399</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>149</v>
+        <v>-117</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>144</v>
+        <v>-115</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -9035,7 +9167,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 40.2% (fair +149). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -9062,22 +9194,22 @@
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays -1.5</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.3698</v>
+        <v>0.4518</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>170</v>
+        <v>121</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -9101,7 +9233,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 37.0% (fair +170). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -9128,22 +9260,22 @@
       </c>
       <c r="D42" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox +1.5</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.6302</v>
+        <v>0.5482</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-170</v>
+        <v>-121</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>178</v>
+        <v>-117</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -9167,7 +9299,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 63.0% (fair -170). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -9184,32 +9316,32 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.4032</v>
+        <v>0.598</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>148</v>
+        <v>-149</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>156</v>
+        <v>100</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -9233,7 +9365,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 40.3% (fair +148). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -9250,32 +9382,32 @@
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D44" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Under 7.5</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.5968</v>
+        <v>0.402</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>-148</v>
+        <v>149</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>-150</v>
+        <v>144</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -9299,7 +9431,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 59.7% (fair -148). Your call.</t>
+          <t>Model 40.2% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -9316,32 +9448,32 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Toronto Blue Jays -1.5</t>
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.4439</v>
+        <v>0.3698</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>125</v>
+        <v>170</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>122</v>
+        <v>164</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -9365,7 +9497,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 37.0% (fair +170). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -9382,32 +9514,32 @@
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C46" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D46" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E46" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Chicago White Sox +1.5</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.5561</v>
+        <v>0.6302</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>-125</v>
+        <v>-170</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-127</v>
+        <v>178</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -9431,7 +9563,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -9448,12 +9580,12 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -9463,17 +9595,17 @@
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4959</v>
+        <v>0.4133</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>102</v>
+        <v>142</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>-108</v>
+        <v>144</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -9497,7 +9629,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 41.3% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -9514,12 +9646,12 @@
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D48" s="20" t="inlineStr">
@@ -9529,17 +9661,17 @@
       </c>
       <c r="E48" s="20" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5041</v>
+        <v>0.5867</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-102</v>
+        <v>-142</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>108</v>
+        <v>-144</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -9563,7 +9695,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -9580,29 +9712,29 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.4933</v>
+        <v>0.4789</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="H49" s="15" t="n">
         <v>104</v>
@@ -9629,7 +9761,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -9646,32 +9778,32 @@
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D50" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.5067</v>
+        <v>0.5211</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-103</v>
+        <v>-109</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -9695,7 +9827,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -9712,32 +9844,32 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>Over 10.5</t>
+          <t>Milwaukee Brewers -1.5</t>
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.4663</v>
+        <v>0.3895</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>114</v>
+        <v>157</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>108</v>
+        <v>152</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -9761,7 +9893,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +114). Your call.</t>
+          <t>Model 39.0% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -9778,32 +9910,32 @@
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D52" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Miami Marlins +1.5</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.5337000000000001</v>
+        <v>0.6105</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>-114</v>
+        <v>-157</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>-104</v>
+        <v>213</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -9827,7 +9959,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -114). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -9844,32 +9976,32 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals +1.5</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.5977</v>
+        <v>0.4332</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>-149</v>
+        <v>131</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>-162</v>
+        <v>127</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -9893,7 +10025,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 59.8% (fair -149). Your call.</t>
+          <t>Model 43.3% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -9910,32 +10042,32 @@
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C54" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D54" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres -1.5</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.4023</v>
+        <v>0.5668</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>149</v>
+        <v>-131</v>
       </c>
       <c r="H54" s="15" t="n">
-        <v>150</v>
+        <v>-127</v>
       </c>
       <c r="I54" s="13">
         <f>IF($H$54="","",IF($H$54&lt;0,-$H$54/(-$H$54+100),100/($H$54+100)))</f>
@@ -9959,7 +10091,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 40.2% (fair +149). Your call.</t>
+          <t>Model 56.7% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -9976,12 +10108,12 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
@@ -9991,16 +10123,18 @@
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.3262</v>
+        <v>0.4959</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>207</v>
-      </c>
-      <c r="H55" s="15" t="n"/>
+        <v>102</v>
+      </c>
+      <c r="H55" s="15" t="n">
+        <v>-108</v>
+      </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
         <v/>
@@ -10023,7 +10157,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 32.6% (fair +207). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -10040,12 +10174,12 @@
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C56" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D56" s="20" t="inlineStr">
@@ -10055,16 +10189,18 @@
       </c>
       <c r="E56" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.6738</v>
+        <v>0.5041</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>-207</v>
-      </c>
-      <c r="H56" s="15" t="n"/>
+        <v>-102</v>
+      </c>
+      <c r="H56" s="15" t="n">
+        <v>108</v>
+      </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
         <v/>
@@ -10087,7 +10223,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 67.4% (fair -207). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -10104,32 +10240,32 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>Over 12.5</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4497</v>
+        <v>0.4985000000000001</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -10153,7 +10289,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 45.0% (fair +122). Your call.</t>
+          <t>Model 49.9% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -10170,32 +10306,32 @@
       </c>
       <c r="B58" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D58" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E58" s="20" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5503</v>
+        <v>0.5014999999999999</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-122</v>
+        <v>-101</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -10219,7 +10355,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 50.1% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -10236,32 +10372,32 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies +1.5</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.6559</v>
+        <v>0.3923</v>
       </c>
       <c r="G59" s="14" t="n">
-        <v>-191</v>
+        <v>155</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>-165</v>
+        <v>108</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -10285,7 +10421,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 65.6% (fair -191). Your call.</t>
+          <t>Model 39.2% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -10302,32 +10438,32 @@
       </c>
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D60" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E60" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds -1.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.3441</v>
+        <v>0.6077</v>
       </c>
       <c r="G60" s="14" t="n">
-        <v>191</v>
+        <v>-155</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -10351,7 +10487,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 34.4% (fair +191). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -10368,31 +10504,33 @@
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ Los Angeles Angels</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Kansas City Royals +1.5</t>
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.5327</v>
+        <v>0.5974</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-114</v>
-      </c>
-      <c r="H61" s="15" t="n"/>
+        <v>-148</v>
+      </c>
+      <c r="H61" s="15" t="n">
+        <v>-156</v>
+      </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
         <v/>
@@ -10415,7 +10553,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 59.7% (fair -148). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -10432,31 +10570,33 @@
       </c>
       <c r="B62" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ Los Angeles Angels</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>San Diego Padres -1.5</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4673</v>
+        <v>0.4026</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>114</v>
-      </c>
-      <c r="H62" s="15" t="n"/>
+        <v>148</v>
+      </c>
+      <c r="H62" s="15" t="n">
+        <v>152</v>
+      </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
         <v/>
@@ -10479,7 +10619,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 40.3% (fair +148). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -10496,12 +10636,12 @@
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Athletics</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
@@ -10511,14 +10651,14 @@
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.5006</v>
+        <v>0.3262</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>-100</v>
+        <v>207</v>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13">
@@ -10543,7 +10683,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 32.6% (fair +207). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -10560,12 +10700,12 @@
       </c>
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Athletics</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D64" s="20" t="inlineStr">
@@ -10575,14 +10715,14 @@
       </c>
       <c r="E64" s="20" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.4995</v>
+        <v>0.6738</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>100</v>
+        <v>-207</v>
       </c>
       <c r="H64" s="15" t="n"/>
       <c r="I64" s="13">
@@ -10607,7 +10747,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair +100). Your call.</t>
+          <t>Model 67.4% (fair -207). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -10624,31 +10764,33 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals</t>
+          <t>Over 12.5</t>
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4814</v>
+        <v>0.4497</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>108</v>
-      </c>
-      <c r="H65" s="15" t="n"/>
+        <v>122</v>
+      </c>
+      <c r="H65" s="15" t="n">
+        <v>117</v>
+      </c>
       <c r="I65" s="13">
         <f>IF($H$65="","",IF($H$65&lt;0,-$H$65/(-$H$65+100),100/($H$65+100)))</f>
         <v/>
@@ -10671,7 +10813,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -10688,31 +10830,33 @@
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D66" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5185999999999999</v>
+        <v>0.5503</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-108</v>
-      </c>
-      <c r="H66" s="15" t="n"/>
+        <v>-122</v>
+      </c>
+      <c r="H66" s="15" t="n">
+        <v>113</v>
+      </c>
       <c r="I66" s="13">
         <f>IF($H$66="","",IF($H$66&lt;0,-$H$66/(-$H$66+100),100/($H$66+100)))</f>
         <v/>
@@ -10735,7 +10879,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -10752,31 +10896,33 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Colorado Rockies -1.5</t>
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>0.4992</v>
+        <v>0.5564</v>
       </c>
       <c r="G67" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="H67" s="15" t="n"/>
+        <v>-125</v>
+      </c>
+      <c r="H67" s="15" t="n">
+        <v>140</v>
+      </c>
       <c r="I67" s="13">
         <f>IF($H$67="","",IF($H$67&lt;0,-$H$67/(-$H$67+100),100/($H$67+100)))</f>
         <v/>
@@ -10799,7 +10945,7 @@
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +100). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O67" s="15" t="n"/>
@@ -10816,31 +10962,33 @@
       </c>
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D68" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E68" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Cincinnati Reds +1.5</t>
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>0.5008</v>
+        <v>0.4436</v>
       </c>
       <c r="G68" s="14" t="n">
-        <v>-100</v>
-      </c>
-      <c r="H68" s="15" t="n"/>
+        <v>125</v>
+      </c>
+      <c r="H68" s="15" t="n">
+        <v>150</v>
+      </c>
       <c r="I68" s="13">
         <f>IF($H$68="","",IF($H$68&lt;0,-$H$68/(-$H$68+100),100/($H$68+100)))</f>
         <v/>
@@ -10863,7 +11011,7 @@
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O68" s="15" t="n"/>
@@ -10872,9 +11020,521 @@
         <v/>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>Detroit Tigers @ Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>01:38</t>
+        </is>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="F69" s="13" t="n">
+        <v>0.5312</v>
+      </c>
+      <c r="G69" s="14" t="n">
+        <v>-113</v>
+      </c>
+      <c r="H69" s="15" t="n"/>
+      <c r="I69" s="13">
+        <f>IF($H$69="","",IF($H$69&lt;0,-$H$69/(-$H$69+100),100/($H$69+100)))</f>
+        <v/>
+      </c>
+      <c r="J69" s="16">
+        <f>IF($H$69="","",$F$69*IF($H$69&lt;0,-100/$H$69,$H$69/100)-(1-$F$69))</f>
+        <v/>
+      </c>
+      <c r="K69" s="17">
+        <f>IF($H$69="","",MAX(0,($F$69*IF($H$69&lt;0,-100/$H$69,$H$69/100)-(1-$F$69))/IF($H$69&lt;0,-100/$H$69,$H$69/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L69" s="18">
+        <f>IF($H$69="","",ROUND(MIN($K$69,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M69" s="12">
+        <f>IF($J$69="","",IF($J$69&lt;0,"Pass",IF($J$69&lt;'Settings'!$B$4,"Thin",IF($J$69&lt;0.06,"✅ Sharp band",IF($J$69&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N69" s="19" t="inlineStr">
+        <is>
+          <t>Model 53.1% (fair -113). Your call.</t>
+        </is>
+      </c>
+      <c r="O69" s="15" t="n"/>
+      <c r="P69" s="16">
+        <f>IF(OR($H$69="",$O$69=""),"",(1+IF($H$69&lt;0,-100/$H$69,$H$69/100))/(1+IF($O$69&lt;0,-100/$O$69,$O$69/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B70" s="20" t="inlineStr">
+        <is>
+          <t>Detroit Tigers @ Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C70" s="20" t="inlineStr">
+        <is>
+          <t>01:38</t>
+        </is>
+      </c>
+      <c r="D70" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E70" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="F70" s="13" t="n">
+        <v>0.4688</v>
+      </c>
+      <c r="G70" s="14" t="n">
+        <v>113</v>
+      </c>
+      <c r="H70" s="15" t="n"/>
+      <c r="I70" s="13">
+        <f>IF($H$70="","",IF($H$70&lt;0,-$H$70/(-$H$70+100),100/($H$70+100)))</f>
+        <v/>
+      </c>
+      <c r="J70" s="16">
+        <f>IF($H$70="","",$F$70*IF($H$70&lt;0,-100/$H$70,$H$70/100)-(1-$F$70))</f>
+        <v/>
+      </c>
+      <c r="K70" s="17">
+        <f>IF($H$70="","",MAX(0,($F$70*IF($H$70&lt;0,-100/$H$70,$H$70/100)-(1-$F$70))/IF($H$70&lt;0,-100/$H$70,$H$70/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L70" s="18">
+        <f>IF($H$70="","",ROUND(MIN($K$70,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M70" s="12">
+        <f>IF($J$70="","",IF($J$70&lt;0,"Pass",IF($J$70&lt;'Settings'!$B$4,"Thin",IF($J$70&lt;0.06,"✅ Sharp band",IF($J$70&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N70" s="19" t="inlineStr">
+        <is>
+          <t>Model 46.9% (fair +113). Your call.</t>
+        </is>
+      </c>
+      <c r="O70" s="15" t="n"/>
+      <c r="P70" s="16">
+        <f>IF(OR($H$70="",$O$70=""),"",(1+IF($H$70&lt;0,-100/$H$70,$H$70/100))/(1+IF($O$70&lt;0,-100/$O$70,$O$70/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>Washington Nationals @ Athletics</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="F71" s="13" t="n">
+        <v>0.5436</v>
+      </c>
+      <c r="G71" s="14" t="n">
+        <v>-119</v>
+      </c>
+      <c r="H71" s="15" t="n"/>
+      <c r="I71" s="13">
+        <f>IF($H$71="","",IF($H$71&lt;0,-$H$71/(-$H$71+100),100/($H$71+100)))</f>
+        <v/>
+      </c>
+      <c r="J71" s="16">
+        <f>IF($H$71="","",$F$71*IF($H$71&lt;0,-100/$H$71,$H$71/100)-(1-$F$71))</f>
+        <v/>
+      </c>
+      <c r="K71" s="17">
+        <f>IF($H$71="","",MAX(0,($F$71*IF($H$71&lt;0,-100/$H$71,$H$71/100)-(1-$F$71))/IF($H$71&lt;0,-100/$H$71,$H$71/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L71" s="18">
+        <f>IF($H$71="","",ROUND(MIN($K$71,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M71" s="12">
+        <f>IF($J$71="","",IF($J$71&lt;0,"Pass",IF($J$71&lt;'Settings'!$B$4,"Thin",IF($J$71&lt;0.06,"✅ Sharp band",IF($J$71&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N71" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.4% (fair -119). Your call.</t>
+        </is>
+      </c>
+      <c r="O71" s="15" t="n"/>
+      <c r="P71" s="16">
+        <f>IF(OR($H$71="",$O$71=""),"",(1+IF($H$71&lt;0,-100/$H$71,$H$71/100))/(1+IF($O$71&lt;0,-100/$O$71,$O$71/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B72" s="20" t="inlineStr">
+        <is>
+          <t>Washington Nationals @ Athletics</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D72" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="F72" s="13" t="n">
+        <v>0.4564</v>
+      </c>
+      <c r="G72" s="14" t="n">
+        <v>119</v>
+      </c>
+      <c r="H72" s="15" t="n"/>
+      <c r="I72" s="13">
+        <f>IF($H$72="","",IF($H$72&lt;0,-$H$72/(-$H$72+100),100/($H$72+100)))</f>
+        <v/>
+      </c>
+      <c r="J72" s="16">
+        <f>IF($H$72="","",$F$72*IF($H$72&lt;0,-100/$H$72,$H$72/100)-(1-$F$72))</f>
+        <v/>
+      </c>
+      <c r="K72" s="17">
+        <f>IF($H$72="","",MAX(0,($F$72*IF($H$72&lt;0,-100/$H$72,$H$72/100)-(1-$F$72))/IF($H$72&lt;0,-100/$H$72,$H$72/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L72" s="18">
+        <f>IF($H$72="","",ROUND(MIN($K$72,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M72" s="12">
+        <f>IF($J$72="","",IF($J$72&lt;0,"Pass",IF($J$72&lt;'Settings'!$B$4,"Thin",IF($J$72&lt;0.06,"✅ Sharp band",IF($J$72&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N72" s="19" t="inlineStr">
+        <is>
+          <t>Model 45.6% (fair +119). Your call.</t>
+        </is>
+      </c>
+      <c r="O72" s="15" t="n"/>
+      <c r="P72" s="16">
+        <f>IF(OR($H$72="",$O$72=""),"",(1+IF($H$72&lt;0,-100/$H$72,$H$72/100))/(1+IF($O$72&lt;0,-100/$O$72,$O$72/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="F73" s="13" t="n">
+        <v>0.4814</v>
+      </c>
+      <c r="G73" s="14" t="n">
+        <v>108</v>
+      </c>
+      <c r="H73" s="15" t="n"/>
+      <c r="I73" s="13">
+        <f>IF($H$73="","",IF($H$73&lt;0,-$H$73/(-$H$73+100),100/($H$73+100)))</f>
+        <v/>
+      </c>
+      <c r="J73" s="16">
+        <f>IF($H$73="","",$F$73*IF($H$73&lt;0,-100/$H$73,$H$73/100)-(1-$F$73))</f>
+        <v/>
+      </c>
+      <c r="K73" s="17">
+        <f>IF($H$73="","",MAX(0,($F$73*IF($H$73&lt;0,-100/$H$73,$H$73/100)-(1-$F$73))/IF($H$73&lt;0,-100/$H$73,$H$73/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L73" s="18">
+        <f>IF($H$73="","",ROUND(MIN($K$73,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M73" s="12">
+        <f>IF($J$73="","",IF($J$73&lt;0,"Pass",IF($J$73&lt;'Settings'!$B$4,"Thin",IF($J$73&lt;0.06,"✅ Sharp band",IF($J$73&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N73" s="19" t="inlineStr">
+        <is>
+          <t>Model 48.1% (fair +108). Your call.</t>
+        </is>
+      </c>
+      <c r="O73" s="15" t="n"/>
+      <c r="P73" s="16">
+        <f>IF(OR($H$73="",$O$73=""),"",(1+IF($H$73&lt;0,-100/$H$73,$H$73/100))/(1+IF($O$73&lt;0,-100/$O$73,$O$73/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B74" s="20" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D74" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="F74" s="13" t="n">
+        <v>0.5185999999999999</v>
+      </c>
+      <c r="G74" s="14" t="n">
+        <v>-108</v>
+      </c>
+      <c r="H74" s="15" t="n"/>
+      <c r="I74" s="13">
+        <f>IF($H$74="","",IF($H$74&lt;0,-$H$74/(-$H$74+100),100/($H$74+100)))</f>
+        <v/>
+      </c>
+      <c r="J74" s="16">
+        <f>IF($H$74="","",$F$74*IF($H$74&lt;0,-100/$H$74,$H$74/100)-(1-$F$74))</f>
+        <v/>
+      </c>
+      <c r="K74" s="17">
+        <f>IF($H$74="","",MAX(0,($F$74*IF($H$74&lt;0,-100/$H$74,$H$74/100)-(1-$F$74))/IF($H$74&lt;0,-100/$H$74,$H$74/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L74" s="18">
+        <f>IF($H$74="","",ROUND(MIN($K$74,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M74" s="12">
+        <f>IF($J$74="","",IF($J$74&lt;0,"Pass",IF($J$74&lt;'Settings'!$B$4,"Thin",IF($J$74&lt;0.06,"✅ Sharp band",IF($J$74&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N74" s="19" t="inlineStr">
+        <is>
+          <t>Model 51.9% (fair -108). Your call.</t>
+        </is>
+      </c>
+      <c r="O74" s="15" t="n"/>
+      <c r="P74" s="16">
+        <f>IF(OR($H$74="",$O$74=""),"",(1+IF($H$74&lt;0,-100/$H$74,$H$74/100))/(1+IF($O$74&lt;0,-100/$O$74,$O$74/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants @ Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="F75" s="13" t="n">
+        <v>0.5033</v>
+      </c>
+      <c r="G75" s="14" t="n">
+        <v>-101</v>
+      </c>
+      <c r="H75" s="15" t="n"/>
+      <c r="I75" s="13">
+        <f>IF($H$75="","",IF($H$75&lt;0,-$H$75/(-$H$75+100),100/($H$75+100)))</f>
+        <v/>
+      </c>
+      <c r="J75" s="16">
+        <f>IF($H$75="","",$F$75*IF($H$75&lt;0,-100/$H$75,$H$75/100)-(1-$F$75))</f>
+        <v/>
+      </c>
+      <c r="K75" s="17">
+        <f>IF($H$75="","",MAX(0,($F$75*IF($H$75&lt;0,-100/$H$75,$H$75/100)-(1-$F$75))/IF($H$75&lt;0,-100/$H$75,$H$75/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L75" s="18">
+        <f>IF($H$75="","",ROUND(MIN($K$75,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M75" s="12">
+        <f>IF($J$75="","",IF($J$75&lt;0,"Pass",IF($J$75&lt;'Settings'!$B$4,"Thin",IF($J$75&lt;0.06,"✅ Sharp band",IF($J$75&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N75" s="19" t="inlineStr">
+        <is>
+          <t>Model 50.3% (fair -101). Your call.</t>
+        </is>
+      </c>
+      <c r="O75" s="15" t="n"/>
+      <c r="P75" s="16">
+        <f>IF(OR($H$75="",$O$75=""),"",(1+IF($H$75&lt;0,-100/$H$75,$H$75/100))/(1+IF($O$75&lt;0,-100/$O$75,$O$75/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B76" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco Giants @ Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="D76" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="F76" s="13" t="n">
+        <v>0.4967</v>
+      </c>
+      <c r="G76" s="14" t="n">
+        <v>101</v>
+      </c>
+      <c r="H76" s="15" t="n"/>
+      <c r="I76" s="13">
+        <f>IF($H$76="","",IF($H$76&lt;0,-$H$76/(-$H$76+100),100/($H$76+100)))</f>
+        <v/>
+      </c>
+      <c r="J76" s="16">
+        <f>IF($H$76="","",$F$76*IF($H$76&lt;0,-100/$H$76,$H$76/100)-(1-$F$76))</f>
+        <v/>
+      </c>
+      <c r="K76" s="17">
+        <f>IF($H$76="","",MAX(0,($F$76*IF($H$76&lt;0,-100/$H$76,$H$76/100)-(1-$F$76))/IF($H$76&lt;0,-100/$H$76,$H$76/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L76" s="18">
+        <f>IF($H$76="","",ROUND(MIN($K$76,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M76" s="12">
+        <f>IF($J$76="","",IF($J$76&lt;0,"Pass",IF($J$76&lt;'Settings'!$B$4,"Thin",IF($J$76&lt;0.06,"✅ Sharp band",IF($J$76&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N76" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.7% (fair +101). Your call.</t>
+        </is>
+      </c>
+      <c r="O76" s="15" t="n"/>
+      <c r="P76" s="16">
+        <f>IF(OR($H$76="",$O$76=""),"",(1+IF($H$76&lt;0,-100/$H$76,$H$76/100))/(1+IF($O$76&lt;0,-100/$O$76,$O$76/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J68">
+  <conditionalFormatting sqref="J5:J76">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -11368,7 +12028,7 @@
         <v>-370</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-115</v>
+        <v>-120</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -11424,17 +12084,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 175.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5814</v>
+        <v>0.5692</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-139</v>
+        <v>-132</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>100</v>
+        <v>-108</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -11458,7 +12118,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 58.1% (fair -139). Your call.</t>
+          <t>Model 56.9% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -11490,17 +12150,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Under 173.5</t>
+          <t>Under 175.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4186</v>
+        <v>0.4308</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -11524,7 +12184,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 41.9% (fair +139). Your call.</t>
+          <t>Model 43.1% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -11824,13 +12484,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5012</v>
+        <v>0.5092</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-100</v>
+        <v>-104</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -11854,7 +12514,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -11890,13 +12550,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4988</v>
+        <v>0.4908</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-105</v>
+        <v>104</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -11920,7 +12580,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +100). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -11956,10 +12616,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.542</v>
+        <v>0.5426</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-118</v>
+        <v>-119</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>108</v>
@@ -11986,7 +12646,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -12022,13 +12682,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.458</v>
+        <v>0.4574</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -12052,7 +12712,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -12088,10 +12748,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4439</v>
+        <v>0.4466</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>108</v>
@@ -12118,7 +12778,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -12154,13 +12814,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5561</v>
+        <v>0.5534</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-125</v>
+        <v>-124</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-113</v>
+        <v>-108</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -12184,7 +12844,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -12216,17 +12876,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Over 185.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5482</v>
+        <v>0.5147</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-121</v>
+        <v>-106</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-105</v>
+        <v>104</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -12250,7 +12910,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -12282,17 +12942,17 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Under 183.5</t>
+          <t>Under 185.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4518</v>
+        <v>0.4853</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -12316,7 +12976,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -12352,13 +13012,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5059</v>
+        <v>0.5013</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-102</v>
+        <v>-101</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -12382,7 +13042,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -102). Your call.</t>
+          <t>Model 50.1% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -12418,13 +13078,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4941</v>
+        <v>0.4987</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -12448,7 +13108,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +102). Your call.</t>
+          <t>Model 49.9% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -12616,10 +13276,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5848</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-141</v>
+        <v>-142</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>-106</v>
@@ -12646,7 +13306,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12682,13 +13342,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4152</v>
+        <v>0.4127999999999999</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -12712,7 +13372,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 41.3% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -12748,10 +13408,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4854</v>
+        <v>0.483</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>-102</v>
@@ -12778,7 +13438,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 48.3% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12814,13 +13474,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5145999999999999</v>
+        <v>0.517</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-106</v>
+        <v>-107</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -12844,7 +13504,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-16 21:12Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-16.xlsx
+++ b/data/output/workbook/2026-07-16.xlsx
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:25</t>
+          <t>2026-07-16 17:12</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6574</v>
+        <v>0.6572</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-192</v>
@@ -5234,10 +5234,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.6094999999999999</v>
+        <v>0.6109</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-156</v>
+        <v>-157</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>156</v>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5347,32 +5347,32 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies -1.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5564</v>
+        <v>0.6535</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-125</v>
+        <v>-189</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 65.3% (fair -189). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -5413,12 +5413,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -5428,17 +5428,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.6559</v>
+        <v>0.6032</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-191</v>
+        <v>-152</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 65.6% (fair -191). Your call.</t>
+          <t>Model 60.3% (fair -152). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -5545,12 +5545,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -5560,17 +5560,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.6077</v>
+        <v>0.598</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-155</v>
+        <v>-149</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -5611,12 +5611,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -5626,17 +5626,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.598</v>
+        <v>0.5631999999999999</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-149</v>
+        <v>-129</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 59.8% (fair -149). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -5677,32 +5677,32 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5729</v>
+        <v>0.4153</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-134</v>
+        <v>141</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -5743,29 +5743,29 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Atlanta Dream @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>Toronto Tempo +6.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5503</v>
+        <v>0.539</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-122</v>
+        <v>-117</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>113</v>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -5809,32 +5809,32 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4153</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>141</v>
+        <v>-142</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>178</v>
+        <v>-106</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -5875,12 +5875,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -5890,17 +5890,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5872000000000001</v>
+        <v>0.5619000000000001</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-142</v>
+        <v>-128</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-106</v>
+        <v>100</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
+          <t>Seattle Storm @ Indiana Fever</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -5951,22 +5951,22 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo +6.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5426</v>
+        <v>0.5802</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-119</v>
+        <v>-138</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>108</v>
+        <v>-108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -6007,32 +6007,32 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds +1.5</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4436</v>
+        <v>0.5338000000000001</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>125</v>
+        <v>-115</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>150</v>
+        <v>106</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
@@ -6083,22 +6083,22 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Over 175.5</t>
+          <t>Chicago Sky</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5692</v>
+        <v>0.5463</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-132</v>
+        <v>-120</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
@@ -6149,22 +6149,22 @@
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5442</v>
+        <v>0.3891</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-119</v>
+        <v>157</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>178</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 38.9% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -6205,12 +6205,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -6220,17 +6220,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.3905</v>
+        <v>0.6587</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>156</v>
+        <v>-193</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>178</v>
+        <v>-156</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -6254,7 +6254,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 65.9% (fair -193). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -6271,32 +6271,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5534</v>
+        <v>0.5306</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-124</v>
+        <v>-113</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -6337,32 +6337,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun +5.5</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.517</v>
+        <v>0.5041</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-107</v>
+        <v>-102</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -6403,12 +6403,12 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -6418,17 +6418,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Over 185.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5147</v>
+        <v>0.5211</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-106</v>
+        <v>-109</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -6469,32 +6469,32 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>New York Yankees +1.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5041</v>
+        <v>0.6344</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-102</v>
+        <v>-174</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>108</v>
+        <v>-156</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 63.4% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -6535,32 +6535,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Connecticut Sun +5.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5026</v>
+        <v>0.5183</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-101</v>
+        <v>-108</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 51.8% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -6601,32 +6601,32 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Texas Rangers +1.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5211</v>
+        <v>0.5399</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-109</v>
+        <v>-117</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 52.1% (fair -109). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -6827,13 +6827,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4547</v>
+        <v>0.4644</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -6857,7 +6857,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.5% (fair +120). Your call.</t>
+          <t>Model 46.4% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -6893,13 +6893,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5453</v>
+        <v>0.5356</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-120</v>
+        <v>-113</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -6945,7 +6945,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -6955,17 +6955,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 10</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4281</v>
+        <v>0.4971</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>117</v>
+        <v>-102</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 42.8% (fair +134). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -7011,7 +7011,7 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -7021,17 +7021,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 10</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4899000000000001</v>
+        <v>0.5029</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>104</v>
+        <v>-101</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-102</v>
+        <v>101</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -7055,7 +7055,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -7077,7 +7077,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -7091,13 +7091,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3735</v>
+        <v>0.3703</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 37.4% (fair +168). Your call.</t>
+          <t>Model 37.0% (fair +170). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -7157,10 +7157,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6265000000000001</v>
+        <v>0.6296999999999999</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-168</v>
+        <v>-170</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>-163</v>
@@ -7187,7 +7187,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 62.7% (fair -168). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -7619,10 +7619,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4230384</v>
+        <v>0.4249418</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>127</v>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5769616</v>
+        <v>0.5750582</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-136</v>
+        <v>-135</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>122</v>
@@ -7715,7 +7715,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -7751,10 +7751,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6559</v>
+        <v>0.6535</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-191</v>
+        <v>-189</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>100</v>
@@ -7781,7 +7781,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 65.6% (fair -191). Your call.</t>
+          <t>Model 65.3% (fair -189). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -7817,10 +7817,10 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3441</v>
+        <v>0.3465</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>144</v>
@@ -7847,7 +7847,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 34.4% (fair +191). Your call.</t>
+          <t>Model 34.7% (fair +189). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -7883,10 +7883,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.3905</v>
+        <v>0.3891</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>178</v>
@@ -7913,7 +7913,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 38.9% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -7949,10 +7949,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.6094999999999999</v>
+        <v>0.6109</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-156</v>
+        <v>-157</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>156</v>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -8015,13 +8015,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4974</v>
+        <v>0.4661999999999999</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-109</v>
+        <v>-108</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -8081,13 +8081,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5026</v>
+        <v>0.5338000000000001</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-101</v>
+        <v>-115</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -8111,7 +8111,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -8147,13 +8147,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4271</v>
+        <v>0.4381</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 42.7% (fair +134). Your call.</t>
+          <t>Model 43.8% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -8213,13 +8213,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5729</v>
+        <v>0.5619000000000001</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-134</v>
+        <v>-128</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -8243,7 +8243,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -8279,10 +8279,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.6066</v>
+        <v>0.6344</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-154</v>
+        <v>-174</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>-156</v>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 60.7% (fair -154). Your call.</t>
+          <t>Model 63.4% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -8345,10 +8345,10 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3934</v>
+        <v>0.3656</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>150</v>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 39.3% (fair +154). Your call.</t>
+          <t>Model 36.6% (fair +174). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -8411,7 +8411,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4617</v>
+        <v>0.4618</v>
       </c>
       <c r="G29" s="14" t="n">
         <v>117</v>
@@ -8477,7 +8477,7 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5383</v>
+        <v>0.5382</v>
       </c>
       <c r="G30" s="14" t="n">
         <v>-117</v>
@@ -8543,10 +8543,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5442</v>
+        <v>0.5306</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-119</v>
+        <v>-113</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>100</v>
@@ -8573,7 +8573,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -8609,10 +8609,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4558</v>
+        <v>0.4694</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -8639,7 +8639,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 46.9% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -8675,13 +8675,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.3426</v>
+        <v>0.3428</v>
       </c>
       <c r="G33" s="14" t="n">
         <v>192</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -8741,7 +8741,7 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.6574</v>
+        <v>0.6572</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>-192</v>
@@ -8939,13 +8939,13 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4909</v>
+        <v>0.4825</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -8969,7 +8969,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 48.2% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -9005,13 +9005,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5091</v>
+        <v>0.5175000000000001</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-104</v>
+        <v>-107</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>-105</v>
+        <v>-115</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -9035,7 +9035,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 51.8% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -9077,7 +9077,7 @@
         <v>117</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -9143,7 +9143,7 @@
         <v>-117</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -9203,10 +9203,10 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.4518</v>
+        <v>0.4487</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H41" s="15" t="n">
         <v>122</v>
@@ -9233,7 +9233,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -9269,13 +9269,13 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5482</v>
+        <v>0.5513</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-121</v>
+        <v>-123</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-117</v>
+        <v>-122</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -9299,7 +9299,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -9473,7 +9473,7 @@
         <v>170</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -9599,13 +9599,13 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4133</v>
+        <v>0.4185</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -9629,7 +9629,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 41.3% (fair +142). Your call.</t>
+          <t>Model 41.9% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -9665,13 +9665,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5867</v>
+        <v>0.5815</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-142</v>
+        <v>-139</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 58.1% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -10259,10 +10259,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4985000000000001</v>
+        <v>0.5006999999999999</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>101</v>
+        <v>-100</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>100</v>
@@ -10289,7 +10289,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +101). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -10325,10 +10325,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5014999999999999</v>
+        <v>0.4993</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-101</v>
+        <v>100</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>100</v>
@@ -10355,7 +10355,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -101). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -10391,10 +10391,10 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.3923</v>
+        <v>0.4368</v>
       </c>
       <c r="G59" s="14" t="n">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="H59" s="15" t="n">
         <v>108</v>
@@ -10421,7 +10421,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 39.2% (fair +155). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -10457,13 +10457,13 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.6077</v>
+        <v>0.5631999999999999</v>
       </c>
       <c r="G60" s="14" t="n">
-        <v>-155</v>
+        <v>-129</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -10487,7 +10487,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -10523,10 +10523,10 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.5974</v>
+        <v>0.5943000000000001</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-148</v>
+        <v>-146</v>
       </c>
       <c r="H61" s="15" t="n">
         <v>-156</v>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 59.7% (fair -148). Your call.</t>
+          <t>Model 59.4% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -10589,13 +10589,13 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4026</v>
+        <v>0.4056999999999999</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -10619,7 +10619,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 40.3% (fair +148). Your call.</t>
+          <t>Model 40.6% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -10655,10 +10655,10 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.3262</v>
+        <v>0.3324</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 32.6% (fair +207). Your call.</t>
+          <t>Model 33.2% (fair +201). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -10719,10 +10719,10 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.6738</v>
+        <v>0.6676</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>-207</v>
+        <v>-201</v>
       </c>
       <c r="H64" s="15" t="n"/>
       <c r="I64" s="13">
@@ -10747,7 +10747,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 67.4% (fair -207). Your call.</t>
+          <t>Model 66.8% (fair -201). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -10783,10 +10783,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4497</v>
+        <v>0.3968</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="H65" s="15" t="n">
         <v>117</v>
@@ -10813,7 +10813,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 45.0% (fair +122). Your call.</t>
+          <t>Model 39.7% (fair +152). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -10849,13 +10849,13 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5503</v>
+        <v>0.6032</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-122</v>
+        <v>-152</v>
       </c>
       <c r="H66" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I66" s="13">
         <f>IF($H$66="","",IF($H$66&lt;0,-$H$66/(-$H$66+100),100/($H$66+100)))</f>
@@ -10879,7 +10879,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 60.3% (fair -152). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -10911,17 +10911,17 @@
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies -1.5</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>0.5564</v>
+        <v>0.6587</v>
       </c>
       <c r="G67" s="14" t="n">
-        <v>-125</v>
+        <v>-193</v>
       </c>
       <c r="H67" s="15" t="n">
-        <v>140</v>
+        <v>-156</v>
       </c>
       <c r="I67" s="13">
         <f>IF($H$67="","",IF($H$67&lt;0,-$H$67/(-$H$67+100),100/($H$67+100)))</f>
@@ -10945,7 +10945,7 @@
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 65.9% (fair -193). Your call.</t>
         </is>
       </c>
       <c r="O67" s="15" t="n"/>
@@ -10977,17 +10977,17 @@
       </c>
       <c r="E68" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds +1.5</t>
+          <t>Cincinnati Reds -1.5</t>
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>0.4436</v>
+        <v>0.3413</v>
       </c>
       <c r="G68" s="14" t="n">
-        <v>125</v>
+        <v>193</v>
       </c>
       <c r="H68" s="15" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I68" s="13">
         <f>IF($H$68="","",IF($H$68&lt;0,-$H$68/(-$H$68+100),100/($H$68+100)))</f>
@@ -11011,7 +11011,7 @@
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 34.1% (fair +193). Your call.</t>
         </is>
       </c>
       <c r="O68" s="15" t="n"/>
@@ -11047,10 +11047,10 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>0.5312</v>
+        <v>0.5327</v>
       </c>
       <c r="G69" s="14" t="n">
-        <v>-113</v>
+        <v>-114</v>
       </c>
       <c r="H69" s="15" t="n"/>
       <c r="I69" s="13">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O69" s="15" t="n"/>
@@ -11111,10 +11111,10 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.4688</v>
+        <v>0.4673</v>
       </c>
       <c r="G70" s="14" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="13">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Model 46.9% (fair +113). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O70" s="15" t="n"/>
@@ -11175,10 +11175,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.5436</v>
+        <v>0.5199</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>-119</v>
+        <v>-108</v>
       </c>
       <c r="H71" s="15" t="n"/>
       <c r="I71" s="13">
@@ -11203,7 +11203,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -11239,10 +11239,10 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.4564</v>
+        <v>0.4801</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="H72" s="15" t="n"/>
       <c r="I72" s="13">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -11431,10 +11431,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.5033</v>
+        <v>0.4734</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>-101</v>
+        <v>111</v>
       </c>
       <c r="H75" s="15" t="n"/>
       <c r="I75" s="13">
@@ -11459,7 +11459,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -11495,10 +11495,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.4967</v>
+        <v>0.5266</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>101</v>
+        <v>-111</v>
       </c>
       <c r="H76" s="15" t="n"/>
       <c r="I76" s="13">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -11962,7 +11962,7 @@
         <v>370</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>355</v>
+        <v>376</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -12084,14 +12084,14 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 175.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5692</v>
+        <v>0.5802</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-132</v>
+        <v>-138</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>-108</v>
@@ -12118,7 +12118,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -12150,14 +12150,14 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Under 175.5</t>
+          <t>Under 174.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4308</v>
+        <v>0.4198</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>104</v>
@@ -12184,7 +12184,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 42.0% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -12220,10 +12220,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4971</v>
+        <v>0.4996</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>104</v>
@@ -12250,7 +12250,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 50.0% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -12286,13 +12286,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5029</v>
+        <v>0.5004</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-101</v>
+        <v>-100</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -12316,7 +12316,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 50.0% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -12484,10 +12484,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5092</v>
+        <v>0.5043</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>100</v>
@@ -12514,7 +12514,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -12550,13 +12550,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4908</v>
+        <v>0.4957</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -12580,7 +12580,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -12616,13 +12616,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5426</v>
+        <v>0.539</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-119</v>
+        <v>-117</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -12646,7 +12646,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -12682,13 +12682,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4574</v>
+        <v>0.461</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -12712,7 +12712,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -12748,13 +12748,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4466</v>
+        <v>0.4537</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -12778,7 +12778,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -12814,13 +12814,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5534</v>
+        <v>0.5463</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-124</v>
+        <v>-120</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -12844,7 +12844,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -12880,10 +12880,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5147</v>
+        <v>0.5391272713322565</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-106</v>
+        <v>-117</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>104</v>
@@ -12910,7 +12910,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -12946,13 +12946,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4853</v>
+        <v>0.4608727286677435</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-104</v>
+        <v>113</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -12976,7 +12976,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -13012,13 +13012,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5013</v>
+        <v>0.4975</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-101</v>
+        <v>101</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -13042,7 +13042,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -101). Your call.</t>
+          <t>Model 49.8% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -13078,13 +13078,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4987</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>101</v>
+        <v>-101</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-108</v>
+        <v>-106</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -13108,7 +13108,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +101). Your call.</t>
+          <t>Model 50.2% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -13408,13 +13408,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.483</v>
+        <v>0.4817</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -13438,7 +13438,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 48.2% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -13474,13 +13474,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.517</v>
+        <v>0.5183</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-107</v>
+        <v>-108</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -13504,7 +13504,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 51.8% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -13687,7 +13687,7 @@
         <v>243</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -13753,7 +13753,7 @@
         <v>130</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -13819,7 +13819,7 @@
         <v>243</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -13951,7 +13951,7 @@
         <v>243</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>570</v>
+        <v>585</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>

</xml_diff>

<commit_message>
data: hourly update 2026-07-16 23:05Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-16.xlsx
+++ b/data/output/workbook/2026-07-16.xlsx
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 17:12</t>
+          <t>2026-07-16 19:05</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5102,13 +5102,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6572</v>
+        <v>0.6562</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-192</v>
+        <v>-191</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 65.7% (fair -192). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5300,10 +5300,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5847</v>
+        <v>0.5887</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-141</v>
+        <v>-143</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>156</v>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -5413,12 +5413,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -5428,17 +5428,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.6032</v>
+        <v>0.6006</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-152</v>
+        <v>-150</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 60.3% (fair -152). Your call.</t>
+          <t>Model 60.1% (fair -150). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -5479,12 +5479,12 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -5498,10 +5498,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.6264999999999999</v>
+        <v>0.598</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-168</v>
+        <v>-149</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>100</v>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 62.6% (fair -168). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -5545,12 +5545,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -5560,17 +5560,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.598</v>
+        <v>0.5509999999999999</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-149</v>
+        <v>-123</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 59.8% (fair -149). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -5677,12 +5677,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Atlanta Dream @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -5692,17 +5692,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Toronto Tempo +6.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4153</v>
+        <v>0.539</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>141</v>
+        <v>-117</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>178</v>
+        <v>113</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -5743,32 +5743,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo +6.5</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.539</v>
+        <v>0.5503</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-117</v>
+        <v>-122</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -5809,32 +5809,32 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5872000000000001</v>
+        <v>0.4113</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-142</v>
+        <v>143</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>-106</v>
+        <v>178</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 41.1% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -5875,12 +5875,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -5890,17 +5890,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5619000000000001</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-128</v>
+        <v>-142</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>100</v>
+        <v>-106</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -5941,32 +5941,32 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 174.5</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5802</v>
+        <v>0.5385</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-138</v>
+        <v>-117</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-108</v>
+        <v>106</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 53.8% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -6007,32 +6007,32 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5338000000000001</v>
+        <v>0.547</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-115</v>
+        <v>-121</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 54.7% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -6224,7 +6224,7 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.6587</v>
+        <v>0.6588000000000001</v>
       </c>
       <c r="G23" s="14" t="n">
         <v>-193</v>
@@ -6271,32 +6271,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Seattle Storm @ Indiana Fever</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Indiana Fever -10.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5306</v>
+        <v>0.4912</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-113</v>
+        <v>104</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -6337,32 +6337,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5041</v>
+        <v>0.5222</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-102</v>
+        <v>-109</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -6403,32 +6403,32 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>New York Yankees +1.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5211</v>
+        <v>0.635</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-109</v>
+        <v>-174</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>100</v>
+        <v>-156</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 52.1% (fair -109). Your call.</t>
+          <t>Model 63.5% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -6469,32 +6469,32 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees +1.5</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.6344</v>
+        <v>0.5077</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-174</v>
+        <v>-103</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-156</v>
+        <v>104</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 63.4% (fair -174). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -6535,32 +6535,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun +5.5</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5183</v>
+        <v>0.5161</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-108</v>
+        <v>-107</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -108). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -6593,75 +6593,9 @@
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>23:15</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>Texas Rangers +1.5</t>
-        </is>
-      </c>
-      <c r="F29" s="13" t="n">
-        <v>0.5399</v>
-      </c>
-      <c r="G29" s="14" t="n">
-        <v>-117</v>
-      </c>
-      <c r="H29" s="15" t="n">
-        <v>-110</v>
-      </c>
-      <c r="I29" s="13">
-        <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
-        <v/>
-      </c>
-      <c r="J29" s="16">
-        <f>IF($H$29="","",$F$29*IF($H$29&lt;0,-100/$H$29,$H$29/100)-(1-$F$29))</f>
-        <v/>
-      </c>
-      <c r="K29" s="17">
-        <f>IF($H$29="","",MAX(0,($F$29*IF($H$29&lt;0,-100/$H$29,$H$29/100)-(1-$F$29))/IF($H$29&lt;0,-100/$H$29,$H$29/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L29" s="18">
-        <f>IF($H$29="","",ROUND(MIN($K$29,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M29" s="12">
-        <f>IF($J$29="","",IF($J$29&lt;0,"Pass",IF($J$29&lt;'Settings'!$B$4,"Thin",IF($J$29&lt;0.06,"✅ Sharp band",IF($J$29&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N29" s="19" t="inlineStr">
-        <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
-        </is>
-      </c>
-      <c r="O29" s="15" t="n"/>
-      <c r="P29" s="16">
-        <f>IF(OR($H$29="",$O$29=""),"",(1+IF($H$29&lt;0,-100/$H$29,$H$29/100))/(1+IF($O$29&lt;0,-100/$O$29,$O$29/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J29">
+  <conditionalFormatting sqref="J5:J28">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -6683,7 +6617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P76"/>
+  <dimension ref="A1:P80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6827,13 +6761,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4644</v>
+        <v>0.4616</v>
       </c>
       <c r="G5" s="14" t="n">
+        <v>117</v>
+      </c>
+      <c r="H5" s="15" t="n">
         <v>115</v>
-      </c>
-      <c r="H5" s="15" t="n">
-        <v>113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -6857,7 +6791,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +115). Your call.</t>
+          <t>Model 46.2% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -6893,13 +6827,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5356</v>
+        <v>0.5384</v>
       </c>
       <c r="G6" s="14" t="n">
+        <v>-117</v>
+      </c>
+      <c r="H6" s="15" t="n">
         <v>-115</v>
-      </c>
-      <c r="H6" s="15" t="n">
-        <v>-113</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -6923,7 +6857,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 53.8% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -6959,13 +6893,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4971</v>
+        <v>0.4959</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-102</v>
+        <v>104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -6989,7 +6923,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -7025,13 +6959,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5029</v>
+        <v>0.5041</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-101</v>
+        <v>-102</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>101</v>
+        <v>-102</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -7055,7 +6989,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -7091,13 +7025,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3703</v>
+        <v>0.3689</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -7121,7 +7055,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 37.0% (fair +170). Your call.</t>
+          <t>Model 36.9% (fair +171). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -7157,10 +7091,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6296999999999999</v>
+        <v>0.6311</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-170</v>
+        <v>-171</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>-163</v>
@@ -7187,7 +7121,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 63.0% (fair -170). Your call.</t>
+          <t>Model 63.1% (fair -171). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -7355,10 +7289,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.6264999999999999</v>
+        <v>0.6006</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-168</v>
+        <v>-150</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>100</v>
@@ -7385,7 +7319,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 62.6% (fair -168). Your call.</t>
+          <t>Model 60.1% (fair -150). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -7421,10 +7355,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3735000000000001</v>
+        <v>0.3994</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>144</v>
@@ -7451,7 +7385,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 37.4% (fair +168). Your call.</t>
+          <t>Model 39.9% (fair +150). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -7487,10 +7421,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4153</v>
+        <v>0.4113</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>178</v>
@@ -7517,7 +7451,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 41.1% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -7553,10 +7487,10 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5847</v>
+        <v>0.5887</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-141</v>
+        <v>-143</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>156</v>
@@ -7583,7 +7517,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8015,10 +7949,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4661999999999999</v>
+        <v>0.4615</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>-108</v>
@@ -8045,7 +7979,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 46.2% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -8081,10 +8015,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5338000000000001</v>
+        <v>0.5385</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-115</v>
+        <v>-117</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>106</v>
@@ -8111,7 +8045,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 53.8% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -8147,10 +8081,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4381</v>
+        <v>0.4778</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>110</v>
@@ -8177,7 +8111,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 43.8% (fair +128). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -8213,10 +8147,10 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5619000000000001</v>
+        <v>0.5222</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-128</v>
+        <v>-109</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>100</v>
@@ -8243,7 +8177,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -8279,7 +8213,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.6344</v>
+        <v>0.635</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>-174</v>
@@ -8309,7 +8243,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 63.4% (fair -174). Your call.</t>
+          <t>Model 63.5% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -8345,7 +8279,7 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3656</v>
+        <v>0.365</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>174</v>
@@ -8375,7 +8309,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 36.6% (fair +174). Your call.</t>
+          <t>Model 36.5% (fair +174). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -8411,13 +8345,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4618</v>
+        <v>0.4588</v>
       </c>
       <c r="G29" s="14" t="n">
+        <v>118</v>
+      </c>
+      <c r="H29" s="15" t="n">
         <v>117</v>
-      </c>
-      <c r="H29" s="15" t="n">
-        <v>113</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -8441,7 +8375,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +117). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -8477,10 +8411,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5382</v>
+        <v>0.5412</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-117</v>
+        <v>-118</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-117</v>
@@ -8507,7 +8441,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -117). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -8543,10 +8477,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5306</v>
+        <v>0.547</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-113</v>
+        <v>-121</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>100</v>
@@ -8573,7 +8507,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 54.7% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -8609,10 +8543,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4694</v>
+        <v>0.453</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -8639,7 +8573,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.9% (fair +113). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -8675,10 +8609,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.3428</v>
+        <v>0.3438</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>180</v>
@@ -8705,7 +8639,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 34.3% (fair +192). Your call.</t>
+          <t>Model 34.4% (fair +191). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -8741,13 +8675,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.6572</v>
+        <v>0.6562</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-192</v>
+        <v>-191</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -8771,7 +8705,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 65.7% (fair -192). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -8939,13 +8873,13 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4825</v>
+        <v>0.4806</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -8969,7 +8903,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 48.2% (fair +107). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -9005,13 +8939,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5175000000000001</v>
+        <v>0.5194</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-107</v>
+        <v>-108</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -9035,7 +8969,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -107). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -9071,10 +9005,10 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.4601</v>
+        <v>0.4555</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H39" s="15" t="n">
         <v>110</v>
@@ -9101,7 +9035,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 45.6% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -9137,13 +9071,13 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5399</v>
+        <v>0.5445</v>
       </c>
       <c r="G40" s="14" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H40" s="15" t="n">
         <v>-117</v>
-      </c>
-      <c r="H40" s="15" t="n">
-        <v>-110</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -9167,7 +9101,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 54.4% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -9731,13 +9665,13 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.4789</v>
+        <v>0.449</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -9761,7 +9695,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 47.9% (fair +109). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -9797,13 +9731,13 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.5211</v>
+        <v>0.5509999999999999</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-109</v>
+        <v>-123</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -9827,7 +9761,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 52.1% (fair -109). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -9869,7 +9803,7 @@
         <v>157</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -10108,32 +10042,32 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.4959</v>
+        <v>0.5161</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>102</v>
+        <v>-107</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>-108</v>
+        <v>-102</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -10157,7 +10091,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -10174,32 +10108,32 @@
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C56" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D56" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E56" s="20" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5041</v>
+        <v>0.4839</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>-102</v>
+        <v>107</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
@@ -10223,7 +10157,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -10240,32 +10174,32 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Chicago Cubs -1.5</t>
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.5006999999999999</v>
+        <v>0.4029</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>-100</v>
+        <v>148</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -10289,7 +10223,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 40.3% (fair +148). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -10306,32 +10240,32 @@
       </c>
       <c r="B58" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D58" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E58" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Minnesota Twins +1.5</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.4993</v>
+        <v>0.5971</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>100</v>
+        <v>-148</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>100</v>
+        <v>-163</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -10355,7 +10289,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +100). Your call.</t>
+          <t>Model 59.7% (fair -148). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -10372,7 +10306,7 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
@@ -10382,22 +10316,22 @@
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>Over 10.5</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.4368</v>
+        <v>0.4923</v>
       </c>
       <c r="G59" s="14" t="n">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>108</v>
+        <v>-108</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -10421,7 +10355,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -10438,7 +10372,7 @@
       </c>
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
@@ -10448,22 +10382,22 @@
       </c>
       <c r="D60" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E60" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.5631999999999999</v>
+        <v>0.5077</v>
       </c>
       <c r="G60" s="14" t="n">
-        <v>-129</v>
+        <v>-103</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -10487,7 +10421,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -10514,22 +10448,22 @@
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals +1.5</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.5943000000000001</v>
+        <v>0.5046999999999999</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-146</v>
+        <v>-102</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>-156</v>
+        <v>-103</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -10553,7 +10487,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 59.4% (fair -146). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -10580,22 +10514,22 @@
       </c>
       <c r="D62" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres -1.5</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4056999999999999</v>
+        <v>0.4953</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>146</v>
+        <v>102</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>150</v>
+        <v>102</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -10619,7 +10553,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 40.6% (fair +146). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -10636,31 +10570,33 @@
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.3324</v>
+        <v>0.4368</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>201</v>
-      </c>
-      <c r="H63" s="15" t="n"/>
+        <v>129</v>
+      </c>
+      <c r="H63" s="15" t="n">
+        <v>108</v>
+      </c>
       <c r="I63" s="13">
         <f>IF($H$63="","",IF($H$63&lt;0,-$H$63/(-$H$63+100),100/($H$63+100)))</f>
         <v/>
@@ -10683,7 +10619,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 33.2% (fair +201). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -10700,31 +10636,33 @@
       </c>
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D64" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E64" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.6676</v>
+        <v>0.5631999999999999</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>-201</v>
-      </c>
-      <c r="H64" s="15" t="n"/>
+        <v>-129</v>
+      </c>
+      <c r="H64" s="15" t="n">
+        <v>107</v>
+      </c>
       <c r="I64" s="13">
         <f>IF($H$64="","",IF($H$64&lt;0,-$H$64/(-$H$64+100),100/($H$64+100)))</f>
         <v/>
@@ -10747,7 +10685,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 66.8% (fair -201). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -10764,32 +10702,32 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>Over 12.5</t>
+          <t>Kansas City Royals +1.5</t>
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.3968</v>
+        <v>0.5943000000000001</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>152</v>
+        <v>-146</v>
       </c>
       <c r="H65" s="15" t="n">
-        <v>117</v>
+        <v>-156</v>
       </c>
       <c r="I65" s="13">
         <f>IF($H$65="","",IF($H$65&lt;0,-$H$65/(-$H$65+100),100/($H$65+100)))</f>
@@ -10813,7 +10751,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 39.7% (fair +152). Your call.</t>
+          <t>Model 59.4% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -10830,32 +10768,32 @@
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D66" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>San Diego Padres -1.5</t>
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.6032</v>
+        <v>0.4056999999999999</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-152</v>
+        <v>146</v>
       </c>
       <c r="H66" s="15" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="I66" s="13">
         <f>IF($H$66="","",IF($H$66&lt;0,-$H$66/(-$H$66+100),100/($H$66+100)))</f>
@@ -10879,7 +10817,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 60.3% (fair -152). Your call.</t>
+          <t>Model 40.6% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -10906,23 +10844,21 @@
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies +1.5</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>0.6587</v>
+        <v>0.3262</v>
       </c>
       <c r="G67" s="14" t="n">
-        <v>-193</v>
-      </c>
-      <c r="H67" s="15" t="n">
-        <v>-156</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="H67" s="15" t="n"/>
       <c r="I67" s="13">
         <f>IF($H$67="","",IF($H$67&lt;0,-$H$67/(-$H$67+100),100/($H$67+100)))</f>
         <v/>
@@ -10945,7 +10881,7 @@
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>Model 65.9% (fair -193). Your call.</t>
+          <t>Model 32.6% (fair +207). Your call.</t>
         </is>
       </c>
       <c r="O67" s="15" t="n"/>
@@ -10972,23 +10908,21 @@
       </c>
       <c r="D68" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E68" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds -1.5</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>0.3413</v>
+        <v>0.6738</v>
       </c>
       <c r="G68" s="14" t="n">
-        <v>193</v>
-      </c>
-      <c r="H68" s="15" t="n">
-        <v>152</v>
-      </c>
+        <v>-207</v>
+      </c>
+      <c r="H68" s="15" t="n"/>
       <c r="I68" s="13">
         <f>IF($H$68="","",IF($H$68&lt;0,-$H$68/(-$H$68+100),100/($H$68+100)))</f>
         <v/>
@@ -11011,7 +10945,7 @@
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>Model 34.1% (fair +193). Your call.</t>
+          <t>Model 67.4% (fair -207). Your call.</t>
         </is>
       </c>
       <c r="O68" s="15" t="n"/>
@@ -11028,31 +10962,33 @@
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ Los Angeles Angels</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E69" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Over 12.5</t>
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>0.5327</v>
+        <v>0.4497</v>
       </c>
       <c r="G69" s="14" t="n">
-        <v>-114</v>
-      </c>
-      <c r="H69" s="15" t="n"/>
+        <v>122</v>
+      </c>
+      <c r="H69" s="15" t="n">
+        <v>117</v>
+      </c>
       <c r="I69" s="13">
         <f>IF($H$69="","",IF($H$69&lt;0,-$H$69/(-$H$69+100),100/($H$69+100)))</f>
         <v/>
@@ -11075,7 +11011,7 @@
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O69" s="15" t="n"/>
@@ -11092,31 +11028,33 @@
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ Los Angeles Angels</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.4673</v>
+        <v>0.5503</v>
       </c>
       <c r="G70" s="14" t="n">
-        <v>114</v>
-      </c>
-      <c r="H70" s="15" t="n"/>
+        <v>-122</v>
+      </c>
+      <c r="H70" s="15" t="n">
+        <v>108</v>
+      </c>
       <c r="I70" s="13">
         <f>IF($H$70="","",IF($H$70&lt;0,-$H$70/(-$H$70+100),100/($H$70+100)))</f>
         <v/>
@@ -11139,7 +11077,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O70" s="15" t="n"/>
@@ -11156,31 +11094,33 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Athletics</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.5199</v>
+        <v>0.6588000000000001</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>-108</v>
-      </c>
-      <c r="H71" s="15" t="n"/>
+        <v>-193</v>
+      </c>
+      <c r="H71" s="15" t="n">
+        <v>-156</v>
+      </c>
       <c r="I71" s="13">
         <f>IF($H$71="","",IF($H$71&lt;0,-$H$71/(-$H$71+100),100/($H$71+100)))</f>
         <v/>
@@ -11203,7 +11143,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 65.9% (fair -193). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -11220,31 +11160,33 @@
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Athletics</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C72" s="20" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D72" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E72" s="20" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Cincinnati Reds -1.5</t>
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.4801</v>
+        <v>0.3411999999999999</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>108</v>
-      </c>
-      <c r="H72" s="15" t="n"/>
+        <v>193</v>
+      </c>
+      <c r="H72" s="15" t="n">
+        <v>154</v>
+      </c>
       <c r="I72" s="13">
         <f>IF($H$72="","",IF($H$72&lt;0,-$H$72/(-$H$72+100),100/($H$72+100)))</f>
         <v/>
@@ -11267,7 +11209,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 34.1% (fair +193). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -11284,12 +11226,12 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Detroit Tigers @ Los Angeles Angels</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>01:38</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
@@ -11299,14 +11241,14 @@
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.4814</v>
+        <v>0.5091</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="H73" s="15" t="n"/>
       <c r="I73" s="13">
@@ -11331,7 +11273,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -11348,12 +11290,12 @@
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Detroit Tigers @ Los Angeles Angels</t>
         </is>
       </c>
       <c r="C74" s="20" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>01:38</t>
         </is>
       </c>
       <c r="D74" s="20" t="inlineStr">
@@ -11363,14 +11305,14 @@
       </c>
       <c r="E74" s="20" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.5185999999999999</v>
+        <v>0.4909</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>-108</v>
+        <v>104</v>
       </c>
       <c r="H74" s="15" t="n"/>
       <c r="I74" s="13">
@@ -11395,7 +11337,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -11412,12 +11354,12 @@
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Washington Nationals @ Athletics</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
@@ -11427,14 +11369,14 @@
       </c>
       <c r="E75" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.4734</v>
+        <v>0.5199</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>111</v>
+        <v>-108</v>
       </c>
       <c r="H75" s="15" t="n"/>
       <c r="I75" s="13">
@@ -11459,7 +11401,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +111). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -11476,12 +11418,12 @@
       </c>
       <c r="B76" s="20" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Washington Nationals @ Athletics</t>
         </is>
       </c>
       <c r="C76" s="20" t="inlineStr">
         <is>
-          <t>02:10</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="D76" s="20" t="inlineStr">
@@ -11491,14 +11433,14 @@
       </c>
       <c r="E76" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.5266</v>
+        <v>0.4801</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-111</v>
+        <v>108</v>
       </c>
       <c r="H76" s="15" t="n"/>
       <c r="I76" s="13">
@@ -11523,7 +11465,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -111). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -11532,9 +11474,265 @@
         <v/>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="F77" s="13" t="n">
+        <v>0.4814</v>
+      </c>
+      <c r="G77" s="14" t="n">
+        <v>108</v>
+      </c>
+      <c r="H77" s="15" t="n"/>
+      <c r="I77" s="13">
+        <f>IF($H$77="","",IF($H$77&lt;0,-$H$77/(-$H$77+100),100/($H$77+100)))</f>
+        <v/>
+      </c>
+      <c r="J77" s="16">
+        <f>IF($H$77="","",$F$77*IF($H$77&lt;0,-100/$H$77,$H$77/100)-(1-$F$77))</f>
+        <v/>
+      </c>
+      <c r="K77" s="17">
+        <f>IF($H$77="","",MAX(0,($F$77*IF($H$77&lt;0,-100/$H$77,$H$77/100)-(1-$F$77))/IF($H$77&lt;0,-100/$H$77,$H$77/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L77" s="18">
+        <f>IF($H$77="","",ROUND(MIN($K$77,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M77" s="12">
+        <f>IF($J$77="","",IF($J$77&lt;0,"Pass",IF($J$77&lt;'Settings'!$B$4,"Thin",IF($J$77&lt;0.06,"✅ Sharp band",IF($J$77&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N77" s="19" t="inlineStr">
+        <is>
+          <t>Model 48.1% (fair +108). Your call.</t>
+        </is>
+      </c>
+      <c r="O77" s="15" t="n"/>
+      <c r="P77" s="16">
+        <f>IF(OR($H$77="",$O$77=""),"",(1+IF($H$77&lt;0,-100/$H$77,$H$77/100))/(1+IF($O$77&lt;0,-100/$O$77,$O$77/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B78" s="20" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="D78" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E78" s="20" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="F78" s="13" t="n">
+        <v>0.5185999999999999</v>
+      </c>
+      <c r="G78" s="14" t="n">
+        <v>-108</v>
+      </c>
+      <c r="H78" s="15" t="n"/>
+      <c r="I78" s="13">
+        <f>IF($H$78="","",IF($H$78&lt;0,-$H$78/(-$H$78+100),100/($H$78+100)))</f>
+        <v/>
+      </c>
+      <c r="J78" s="16">
+        <f>IF($H$78="","",$F$78*IF($H$78&lt;0,-100/$H$78,$H$78/100)-(1-$F$78))</f>
+        <v/>
+      </c>
+      <c r="K78" s="17">
+        <f>IF($H$78="","",MAX(0,($F$78*IF($H$78&lt;0,-100/$H$78,$H$78/100)-(1-$F$78))/IF($H$78&lt;0,-100/$H$78,$H$78/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L78" s="18">
+        <f>IF($H$78="","",ROUND(MIN($K$78,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M78" s="12">
+        <f>IF($J$78="","",IF($J$78&lt;0,"Pass",IF($J$78&lt;'Settings'!$B$4,"Thin",IF($J$78&lt;0.06,"✅ Sharp band",IF($J$78&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N78" s="19" t="inlineStr">
+        <is>
+          <t>Model 51.9% (fair -108). Your call.</t>
+        </is>
+      </c>
+      <c r="O78" s="15" t="n"/>
+      <c r="P78" s="16">
+        <f>IF(OR($H$78="",$O$78=""),"",(1+IF($H$78&lt;0,-100/$H$78,$H$78/100))/(1+IF($O$78&lt;0,-100/$O$78,$O$78/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants @ Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="F79" s="13" t="n">
+        <v>0.4734</v>
+      </c>
+      <c r="G79" s="14" t="n">
+        <v>111</v>
+      </c>
+      <c r="H79" s="15" t="n"/>
+      <c r="I79" s="13">
+        <f>IF($H$79="","",IF($H$79&lt;0,-$H$79/(-$H$79+100),100/($H$79+100)))</f>
+        <v/>
+      </c>
+      <c r="J79" s="16">
+        <f>IF($H$79="","",$F$79*IF($H$79&lt;0,-100/$H$79,$H$79/100)-(1-$F$79))</f>
+        <v/>
+      </c>
+      <c r="K79" s="17">
+        <f>IF($H$79="","",MAX(0,($F$79*IF($H$79&lt;0,-100/$H$79,$H$79/100)-(1-$F$79))/IF($H$79&lt;0,-100/$H$79,$H$79/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L79" s="18">
+        <f>IF($H$79="","",ROUND(MIN($K$79,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M79" s="12">
+        <f>IF($J$79="","",IF($J$79&lt;0,"Pass",IF($J$79&lt;'Settings'!$B$4,"Thin",IF($J$79&lt;0.06,"✅ Sharp band",IF($J$79&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N79" s="19" t="inlineStr">
+        <is>
+          <t>Model 47.3% (fair +111). Your call.</t>
+        </is>
+      </c>
+      <c r="O79" s="15" t="n"/>
+      <c r="P79" s="16">
+        <f>IF(OR($H$79="",$O$79=""),"",(1+IF($H$79&lt;0,-100/$H$79,$H$79/100))/(1+IF($O$79&lt;0,-100/$O$79,$O$79/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B80" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco Giants @ Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C80" s="20" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="D80" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E80" s="20" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="n">
+        <v>0.5266</v>
+      </c>
+      <c r="G80" s="14" t="n">
+        <v>-111</v>
+      </c>
+      <c r="H80" s="15" t="n"/>
+      <c r="I80" s="13">
+        <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
+        <v/>
+      </c>
+      <c r="J80" s="16">
+        <f>IF($H$80="","",$F$80*IF($H$80&lt;0,-100/$H$80,$H$80/100)-(1-$F$80))</f>
+        <v/>
+      </c>
+      <c r="K80" s="17">
+        <f>IF($H$80="","",MAX(0,($F$80*IF($H$80&lt;0,-100/$H$80,$H$80/100)-(1-$F$80))/IF($H$80&lt;0,-100/$H$80,$H$80/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L80" s="18">
+        <f>IF($H$80="","",ROUND(MIN($K$80,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M80" s="12">
+        <f>IF($J$80="","",IF($J$80&lt;0,"Pass",IF($J$80&lt;'Settings'!$B$4,"Thin",IF($J$80&lt;0.06,"✅ Sharp band",IF($J$80&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N80" s="19" t="inlineStr">
+        <is>
+          <t>Model 52.7% (fair -111). Your call.</t>
+        </is>
+      </c>
+      <c r="O80" s="15" t="n"/>
+      <c r="P80" s="16">
+        <f>IF(OR($H$80="",$O$80=""),"",(1+IF($H$80&lt;0,-100/$H$80,$H$80/100))/(1+IF($O$80&lt;0,-100/$O$80,$O$80/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J76">
+  <conditionalFormatting sqref="J5:J80">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -11962,7 +12160,7 @@
         <v>370</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>376</v>
+        <v>355</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -12084,17 +12282,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 174.5</t>
+          <t>Over 176.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5802</v>
+        <v>0.6014333181500525</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-138</v>
+        <v>-151</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-108</v>
+        <v>117</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -12118,7 +12316,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 60.1% (fair -151). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -12150,17 +12348,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Under 174.5</t>
+          <t>Under 176.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4198</v>
+        <v>0.3985666818499475</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -12184,7 +12382,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 39.9% (fair +151). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -12220,13 +12418,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4996</v>
+        <v>0.4912</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -12250,7 +12448,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair +100). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -12286,13 +12484,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5004</v>
+        <v>0.5087999999999999</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-100</v>
+        <v>-104</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>-105</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -12316,7 +12514,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair -100). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -12358,7 +12556,7 @@
         <v>-209</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -12484,10 +12682,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5043</v>
+        <v>0.5079</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>100</v>
@@ -12514,7 +12712,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -12550,13 +12748,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4957</v>
+        <v>0.4921</v>
       </c>
       <c r="G18" s="14" t="n">
+        <v>103</v>
+      </c>
+      <c r="H18" s="15" t="n">
         <v>102</v>
-      </c>
-      <c r="H18" s="15" t="n">
-        <v>-104</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -12580,7 +12778,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -13012,13 +13210,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4975</v>
+        <v>0.5072245440157978</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>101</v>
+        <v>-103</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -13042,7 +13240,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -13078,13 +13276,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5024999999999999</v>
+        <v>0.4927754559842022</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-101</v>
+        <v>103</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-106</v>
+        <v>-102</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -13108,7 +13306,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -13216,7 +13414,7 @@
         <v>-150</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -13408,13 +13606,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4817</v>
+        <v>0.4586096690524682</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-104</v>
+        <v>110</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -13438,7 +13636,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 48.2% (fair +108). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -13474,10 +13672,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5183</v>
+        <v>0.5413903309475318</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-108</v>
+        <v>-118</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -13504,7 +13702,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -108). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -13537,7 +13735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13687,7 +13885,7 @@
         <v>243</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -13753,7 +13951,7 @@
         <v>130</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -13794,7 +13992,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Vancouver Whitecaps @ Chicago Fire FC</t>
+          <t>Sporting Kansas City @ St. Louis CITY SC</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -13809,7 +14007,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Vancouver Whitecaps</t>
+          <t>Sporting Kansas City</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
@@ -13819,7 +14017,7 @@
         <v>243</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>155</v>
+        <v>585</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -13860,7 +14058,7 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Vancouver Whitecaps @ Chicago Fire FC</t>
+          <t>Sporting Kansas City @ St. Louis CITY SC</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -13875,7 +14073,7 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Chicago Fire FC</t>
+          <t>St. Louis CITY SC</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
@@ -13885,7 +14083,7 @@
         <v>130</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>165</v>
+        <v>-220</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -13926,12 +14124,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Sporting Kansas City @ St. Louis CITY SC</t>
+          <t>Portland Timbers @ Seattle Sounders FC</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -13941,7 +14139,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Sporting Kansas City</t>
+          <t>Portland Timbers</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
@@ -13951,7 +14149,7 @@
         <v>243</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>585</v>
+        <v>500</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -13992,12 +14190,12 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Sporting Kansas City @ St. Louis CITY SC</t>
+          <t>Portland Timbers @ Seattle Sounders FC</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -14007,7 +14205,7 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>St. Louis CITY SC</t>
+          <t>Seattle Sounders FC</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
@@ -14017,7 +14215,7 @@
         <v>130</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-220</v>
+        <v>-200</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -14053,17 +14251,17 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Portland Timbers @ Seattle Sounders FC</t>
+          <t>Atlanta United FC @ Nashville SC</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -14073,7 +14271,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Portland Timbers</t>
+          <t>Atlanta United FC</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
@@ -14083,7 +14281,7 @@
         <v>243</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -14119,17 +14317,17 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Portland Timbers @ Seattle Sounders FC</t>
+          <t>Atlanta United FC @ Nashville SC</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -14139,7 +14337,7 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Seattle Sounders FC</t>
+          <t>Nashville SC</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
@@ -14190,12 +14388,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Atlanta United FC @ Nashville SC</t>
+          <t>LAFC @ LA Galaxy</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>02:25</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -14205,7 +14403,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Atlanta United FC</t>
+          <t>LAFC</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
@@ -14214,9 +14412,7 @@
       <c r="G13" s="14" t="n">
         <v>243</v>
       </c>
-      <c r="H13" s="15" t="n">
-        <v>600</v>
-      </c>
+      <c r="H13" s="15" t="n"/>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
         <v/>
@@ -14256,12 +14452,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Atlanta United FC @ Nashville SC</t>
+          <t>LAFC @ LA Galaxy</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>02:25</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -14271,7 +14467,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Nashville SC</t>
+          <t>LA Galaxy</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
@@ -14280,9 +14476,7 @@
       <c r="G14" s="14" t="n">
         <v>130</v>
       </c>
-      <c r="H14" s="15" t="n">
-        <v>-210</v>
-      </c>
+      <c r="H14" s="15" t="n"/>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
         <v/>
@@ -14314,137 +14508,9 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>LAFC @ LA Galaxy</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>02:25</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>LAFC</t>
-        </is>
-      </c>
-      <c r="F15" s="13" t="n">
-        <v>0.2919</v>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>243</v>
-      </c>
-      <c r="H15" s="15" t="n"/>
-      <c r="I15" s="13">
-        <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
-        <v/>
-      </c>
-      <c r="J15" s="16">
-        <f>IF($H$15="","",$F$15*IF($H$15&lt;0,-100/$H$15,$H$15/100)-(1-$F$15))</f>
-        <v/>
-      </c>
-      <c r="K15" s="17">
-        <f>IF($H$15="","",MAX(0,($F$15*IF($H$15&lt;0,-100/$H$15,$H$15/100)-(1-$F$15))/IF($H$15&lt;0,-100/$H$15,$H$15/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L15" s="18">
-        <f>IF($H$15="","",ROUND(MIN($K$15,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M15" s="12">
-        <f>IF($J$15="","",IF($J$15&lt;0,"Pass",IF($J$15&lt;'Settings'!$B$4,"Thin",IF($J$15&lt;0.06,"✅ Sharp band",IF($J$15&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N15" s="19" t="inlineStr">
-        <is>
-          <t>Model 29.2% (fair +243). Your call.</t>
-        </is>
-      </c>
-      <c r="O15" s="15" t="n"/>
-      <c r="P15" s="16">
-        <f>IF(OR($H$15="",$O$15=""),"",(1+IF($H$15&lt;0,-100/$H$15,$H$15/100))/(1+IF($O$15&lt;0,-100/$O$15,$O$15/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>LAFC @ LA Galaxy</t>
-        </is>
-      </c>
-      <c r="C16" s="20" t="inlineStr">
-        <is>
-          <t>02:25</t>
-        </is>
-      </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>LA Galaxy</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0.4342</v>
-      </c>
-      <c r="G16" s="14" t="n">
-        <v>130</v>
-      </c>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="13">
-        <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
-        <v/>
-      </c>
-      <c r="J16" s="16">
-        <f>IF($H$16="","",$F$16*IF($H$16&lt;0,-100/$H$16,$H$16/100)-(1-$F$16))</f>
-        <v/>
-      </c>
-      <c r="K16" s="17">
-        <f>IF($H$16="","",MAX(0,($F$16*IF($H$16&lt;0,-100/$H$16,$H$16/100)-(1-$F$16))/IF($H$16&lt;0,-100/$H$16,$H$16/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L16" s="18">
-        <f>IF($H$16="","",ROUND(MIN($K$16,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M16" s="12">
-        <f>IF($J$16="","",IF($J$16&lt;0,"Pass",IF($J$16&lt;'Settings'!$B$4,"Thin",IF($J$16&lt;0.06,"✅ Sharp band",IF($J$16&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N16" s="19" t="inlineStr">
-        <is>
-          <t>Model 43.4% (fair +130). Your call.</t>
-        </is>
-      </c>
-      <c r="O16" s="15" t="n"/>
-      <c r="P16" s="16">
-        <f>IF(OR($H$16="",$O$16=""),"",(1+IF($H$16&lt;0,-100/$H$16,$H$16/100))/(1+IF($O$16&lt;0,-100/$O$16,$O$16/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J16">
+  <conditionalFormatting sqref="J5:J14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>